<commit_message>
Working with trust center
</commit_message>
<xml_diff>
--- a/Input List/Full Band/Input List.xlsx
+++ b/Input List/Full Band/Input List.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27726"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Dev\TechnicalDocumentation\Input List\Full Band\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Dev\TechnicalDocumentation\Input List\Full Band\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF833D77-0232-45E5-999F-C3D6C9CA850C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22EF32D0-0A49-4F7D-806F-B0910D7864BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25180" windowHeight="16140" activeTab="1" xr2:uid="{976BA9A3-41FE-45E5-BC0B-B40312D9AF21}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{976BA9A3-41FE-45E5-BC0B-B40312D9AF21}"/>
   </bookViews>
   <sheets>
     <sheet name="Input + Equipment" sheetId="1" r:id="rId1"/>
@@ -799,37 +799,33 @@
     <xf numFmtId="0" fontId="4" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="12" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -855,29 +851,110 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="12" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="12" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -891,88 +968,11 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="13" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1367,21 +1367,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{18A11D25-D77D-4358-9E34-E04B11CA4C7B}">
   <dimension ref="A1:I35"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.81640625" customWidth="1"/>
-    <col min="2" max="2" width="8.7265625" customWidth="1"/>
-    <col min="3" max="3" width="8.26953125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="6.26953125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.85546875" customWidth="1"/>
+    <col min="2" max="2" width="8.7109375" customWidth="1"/>
+    <col min="3" max="3" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="6.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="15" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="19.453125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.81640625" customWidth="1"/>
-    <col min="8" max="8" width="4.1796875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="34.453125" customWidth="1"/>
-    <col min="10" max="12" width="7.26953125" customWidth="1"/>
+    <col min="6" max="6" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.85546875" customWidth="1"/>
+    <col min="8" max="8" width="4.140625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="34.42578125" customWidth="1"/>
+    <col min="10" max="12" width="7.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="33" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
@@ -1398,7 +1398,7 @@
       <c r="H1" s="35"/>
       <c r="I1" s="35"/>
     </row>
-    <row r="2" spans="1:9" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="34"/>
       <c r="B2" s="34"/>
       <c r="C2" s="38"/>
@@ -1409,7 +1409,7 @@
       <c r="H2" s="36"/>
       <c r="I2" s="36"/>
     </row>
-    <row r="3" spans="1:9" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="9" t="s">
         <v>49</v>
       </c>
@@ -1438,253 +1438,253 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="69" t="s">
+    <row r="4" spans="1:9" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="39" t="s">
         <v>50</v>
       </c>
-      <c r="B4" s="70" t="s">
+      <c r="B4" s="42" t="s">
         <v>30</v>
       </c>
-      <c r="C4" s="71">
+      <c r="C4" s="21">
         <v>1</v>
       </c>
-      <c r="D4" s="71">
+      <c r="D4" s="21">
         <v>1</v>
       </c>
-      <c r="E4" s="71" t="s">
+      <c r="E4" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="F4" s="71" t="s">
+      <c r="F4" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="G4" s="71" t="s">
+      <c r="G4" s="21" t="s">
         <v>79</v>
       </c>
-      <c r="H4" s="71"/>
-      <c r="I4" s="71" t="s">
+      <c r="H4" s="21"/>
+      <c r="I4" s="21" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="72"/>
-      <c r="B5" s="73"/>
-      <c r="C5" s="74">
+    <row r="5" spans="1:9" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="40"/>
+      <c r="B5" s="43"/>
+      <c r="C5" s="22">
         <v>2</v>
       </c>
-      <c r="D5" s="74">
+      <c r="D5" s="22">
         <v>2</v>
       </c>
-      <c r="E5" s="74" t="s">
+      <c r="E5" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="F5" s="74" t="s">
+      <c r="F5" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="G5" s="74" t="s">
+      <c r="G5" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="H5" s="74"/>
-      <c r="I5" s="74" t="s">
+      <c r="H5" s="22"/>
+      <c r="I5" s="22" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="72"/>
-      <c r="B6" s="73"/>
-      <c r="C6" s="71">
+    <row r="6" spans="1:9" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="40"/>
+      <c r="B6" s="43"/>
+      <c r="C6" s="21">
         <v>3</v>
       </c>
-      <c r="D6" s="71">
+      <c r="D6" s="21">
         <v>3</v>
       </c>
-      <c r="E6" s="71" t="s">
+      <c r="E6" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="F6" s="71" t="s">
+      <c r="F6" s="21" t="s">
         <v>26</v>
       </c>
-      <c r="G6" s="71" t="s">
+      <c r="G6" s="21" t="s">
         <v>78</v>
       </c>
-      <c r="H6" s="71"/>
-      <c r="I6" s="71"/>
-    </row>
-    <row r="7" spans="1:9" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="72"/>
-      <c r="B7" s="73"/>
-      <c r="C7" s="74">
+      <c r="H6" s="21"/>
+      <c r="I6" s="21"/>
+    </row>
+    <row r="7" spans="1:9" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="40"/>
+      <c r="B7" s="43"/>
+      <c r="C7" s="22">
         <v>4</v>
       </c>
-      <c r="D7" s="74">
+      <c r="D7" s="22">
         <v>4</v>
       </c>
-      <c r="E7" s="74" t="s">
+      <c r="E7" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="F7" s="74" t="s">
+      <c r="F7" s="22" t="s">
         <v>29</v>
       </c>
-      <c r="G7" s="74" t="s">
+      <c r="G7" s="22" t="s">
         <v>78</v>
       </c>
-      <c r="H7" s="74" t="s">
+      <c r="H7" s="22" t="s">
         <v>38</v>
       </c>
-      <c r="I7" s="74" t="s">
+      <c r="I7" s="22" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="72"/>
-      <c r="B8" s="73"/>
-      <c r="C8" s="71">
+    <row r="8" spans="1:9" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="40"/>
+      <c r="B8" s="43"/>
+      <c r="C8" s="21">
         <v>5</v>
       </c>
-      <c r="D8" s="71">
+      <c r="D8" s="21">
         <v>5</v>
       </c>
-      <c r="E8" s="71" t="s">
+      <c r="E8" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="F8" s="71" t="s">
+      <c r="F8" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="G8" s="71" t="s">
+      <c r="G8" s="21" t="s">
         <v>78</v>
       </c>
-      <c r="H8" s="71" t="s">
+      <c r="H8" s="21" t="s">
         <v>38</v>
       </c>
-      <c r="I8" s="71" t="s">
+      <c r="I8" s="21" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="72"/>
-      <c r="B9" s="73"/>
-      <c r="C9" s="74">
+    <row r="9" spans="1:9" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="40"/>
+      <c r="B9" s="43"/>
+      <c r="C9" s="22">
         <v>6</v>
       </c>
-      <c r="D9" s="74">
+      <c r="D9" s="22">
         <v>6</v>
       </c>
-      <c r="E9" s="74" t="s">
+      <c r="E9" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="F9" s="74" t="s">
+      <c r="F9" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="G9" s="74" t="s">
+      <c r="G9" s="22" t="s">
         <v>78</v>
       </c>
-      <c r="H9" s="74" t="s">
+      <c r="H9" s="22" t="s">
         <v>38</v>
       </c>
-      <c r="I9" s="74" t="s">
+      <c r="I9" s="22" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="72"/>
-      <c r="B10" s="73"/>
-      <c r="C10" s="71">
+    <row r="10" spans="1:9" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="40"/>
+      <c r="B10" s="43"/>
+      <c r="C10" s="21">
         <v>7</v>
       </c>
-      <c r="D10" s="71">
+      <c r="D10" s="21">
         <v>7</v>
       </c>
-      <c r="E10" s="71" t="s">
+      <c r="E10" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="F10" s="71" t="s">
+      <c r="F10" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="G10" s="71" t="s">
+      <c r="G10" s="21" t="s">
         <v>78</v>
       </c>
-      <c r="H10" s="71" t="s">
+      <c r="H10" s="21" t="s">
         <v>38</v>
       </c>
-      <c r="I10" s="71" t="s">
+      <c r="I10" s="21" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="11" spans="1:9" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="72"/>
-      <c r="B11" s="73"/>
-      <c r="C11" s="74">
+    <row r="11" spans="1:9" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="40"/>
+      <c r="B11" s="43"/>
+      <c r="C11" s="22">
         <v>8</v>
       </c>
-      <c r="D11" s="74">
+      <c r="D11" s="22">
         <v>8</v>
       </c>
-      <c r="E11" s="74" t="s">
+      <c r="E11" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="F11" s="74" t="s">
+      <c r="F11" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="G11" s="74" t="s">
+      <c r="G11" s="22" t="s">
         <v>78</v>
       </c>
-      <c r="H11" s="74" t="s">
+      <c r="H11" s="22" t="s">
         <v>38</v>
       </c>
-      <c r="I11" s="74" t="s">
+      <c r="I11" s="22" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="12" spans="1:9" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A12" s="72"/>
-      <c r="B12" s="73"/>
-      <c r="C12" s="71">
+    <row r="12" spans="1:9" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="40"/>
+      <c r="B12" s="43"/>
+      <c r="C12" s="21">
         <v>9</v>
       </c>
-      <c r="D12" s="71">
+      <c r="D12" s="21">
         <v>9</v>
       </c>
-      <c r="E12" s="71" t="s">
+      <c r="E12" s="21" t="s">
         <v>52</v>
       </c>
-      <c r="F12" s="71" t="s">
+      <c r="F12" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="G12" s="71" t="s">
+      <c r="G12" s="21" t="s">
         <v>80</v>
       </c>
-      <c r="H12" s="71" t="s">
+      <c r="H12" s="21" t="s">
         <v>38</v>
       </c>
-      <c r="I12" s="71" t="s">
+      <c r="I12" s="21" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="13" spans="1:9" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="75"/>
-      <c r="B13" s="76"/>
-      <c r="C13" s="74">
+    <row r="13" spans="1:9" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="41"/>
+      <c r="B13" s="44"/>
+      <c r="C13" s="22">
         <v>10</v>
       </c>
-      <c r="D13" s="74">
+      <c r="D13" s="22">
         <v>10</v>
       </c>
-      <c r="E13" s="74" t="s">
+      <c r="E13" s="22" t="s">
         <v>51</v>
       </c>
-      <c r="F13" s="74" t="s">
+      <c r="F13" s="22" t="s">
         <v>29</v>
       </c>
-      <c r="G13" s="74" t="s">
+      <c r="G13" s="22" t="s">
         <v>80</v>
       </c>
-      <c r="H13" s="74" t="s">
+      <c r="H13" s="22" t="s">
         <v>38</v>
       </c>
-      <c r="I13" s="74" t="s">
+      <c r="I13" s="22" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="14" spans="1:9" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="15"/>
       <c r="B14" s="15"/>
       <c r="C14" s="4">
@@ -1693,15 +1693,15 @@
       <c r="D14" s="4">
         <v>11</v>
       </c>
-      <c r="E14" s="21" t="s">
+      <c r="E14" s="25" t="s">
         <v>31</v>
       </c>
-      <c r="F14" s="21"/>
-      <c r="G14" s="21"/>
-      <c r="H14" s="21"/>
-      <c r="I14" s="21"/>
-    </row>
-    <row r="15" spans="1:9" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="F14" s="25"/>
+      <c r="G14" s="25"/>
+      <c r="H14" s="25"/>
+      <c r="I14" s="25"/>
+    </row>
+    <row r="15" spans="1:9" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="15"/>
       <c r="B15" s="15"/>
       <c r="C15" s="4">
@@ -1710,15 +1710,15 @@
       <c r="D15" s="4">
         <v>12</v>
       </c>
-      <c r="E15" s="21" t="s">
+      <c r="E15" s="25" t="s">
         <v>31</v>
       </c>
-      <c r="F15" s="21"/>
-      <c r="G15" s="21"/>
-      <c r="H15" s="21"/>
-      <c r="I15" s="21"/>
-    </row>
-    <row r="16" spans="1:9" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="F15" s="25"/>
+      <c r="G15" s="25"/>
+      <c r="H15" s="25"/>
+      <c r="I15" s="25"/>
+    </row>
+    <row r="16" spans="1:9" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="15"/>
       <c r="B16" s="15"/>
       <c r="C16" s="4">
@@ -1727,15 +1727,15 @@
       <c r="D16" s="4">
         <v>13</v>
       </c>
-      <c r="E16" s="21" t="s">
+      <c r="E16" s="25" t="s">
         <v>31</v>
       </c>
-      <c r="F16" s="21"/>
-      <c r="G16" s="21"/>
-      <c r="H16" s="21"/>
-      <c r="I16" s="21"/>
-    </row>
-    <row r="17" spans="1:9" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="F16" s="25"/>
+      <c r="G16" s="25"/>
+      <c r="H16" s="25"/>
+      <c r="I16" s="25"/>
+    </row>
+    <row r="17" spans="1:9" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="15"/>
       <c r="B17" s="15"/>
       <c r="C17" s="4">
@@ -1744,16 +1744,16 @@
       <c r="D17" s="4">
         <v>14</v>
       </c>
-      <c r="E17" s="21" t="s">
+      <c r="E17" s="25" t="s">
         <v>31</v>
       </c>
-      <c r="F17" s="21"/>
-      <c r="G17" s="21"/>
-      <c r="H17" s="21"/>
-      <c r="I17" s="21"/>
-    </row>
-    <row r="18" spans="1:9" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="39" t="s">
+      <c r="F17" s="25"/>
+      <c r="G17" s="25"/>
+      <c r="H17" s="25"/>
+      <c r="I17" s="25"/>
+    </row>
+    <row r="18" spans="1:9" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="23" t="s">
         <v>62</v>
       </c>
       <c r="B18" s="32" t="s">
@@ -1777,8 +1777,8 @@
       <c r="H18" s="2"/>
       <c r="I18" s="2"/>
     </row>
-    <row r="19" spans="1:9" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="39"/>
+    <row r="19" spans="1:9" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="23"/>
       <c r="B19" s="32"/>
       <c r="C19" s="12">
         <v>16</v>
@@ -1798,11 +1798,11 @@
       <c r="H19" s="12"/>
       <c r="I19" s="12"/>
     </row>
-    <row r="20" spans="1:9" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="26" t="s">
+    <row r="20" spans="1:9" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="49" t="s">
         <v>92</v>
       </c>
-      <c r="B20" s="28" t="s">
+      <c r="B20" s="51" t="s">
         <v>96</v>
       </c>
       <c r="C20" s="13">
@@ -1825,9 +1825,9 @@
         <v>81</v>
       </c>
     </row>
-    <row r="21" spans="1:9" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A21" s="27"/>
-      <c r="B21" s="29"/>
+    <row r="21" spans="1:9" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="50"/>
+      <c r="B21" s="52"/>
       <c r="C21" s="14">
         <v>18</v>
       </c>
@@ -1846,9 +1846,9 @@
       <c r="H21" s="14"/>
       <c r="I21" s="14"/>
     </row>
-    <row r="22" spans="1:9" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="27"/>
-      <c r="B22" s="29"/>
+    <row r="22" spans="1:9" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="50"/>
+      <c r="B22" s="52"/>
       <c r="C22" s="13">
         <v>19</v>
       </c>
@@ -1867,11 +1867,11 @@
       <c r="H22" s="13"/>
       <c r="I22" s="13"/>
     </row>
-    <row r="23" spans="1:9" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="30" t="s">
+    <row r="23" spans="1:9" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="53" t="s">
         <v>93</v>
       </c>
-      <c r="B23" s="31" t="s">
+      <c r="B23" s="54" t="s">
         <v>98</v>
       </c>
       <c r="C23" s="7">
@@ -1894,9 +1894,9 @@
         <v>82</v>
       </c>
     </row>
-    <row r="24" spans="1:9" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A24" s="30"/>
-      <c r="B24" s="31"/>
+    <row r="24" spans="1:9" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="53"/>
+      <c r="B24" s="54"/>
       <c r="C24" s="8">
         <v>21</v>
       </c>
@@ -1915,11 +1915,11 @@
       <c r="H24" s="8"/>
       <c r="I24" s="8"/>
     </row>
-    <row r="25" spans="1:9" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A25" s="22" t="s">
+    <row r="25" spans="1:9" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="45" t="s">
         <v>94</v>
       </c>
-      <c r="B25" s="24" t="s">
+      <c r="B25" s="47" t="s">
         <v>99</v>
       </c>
       <c r="C25" s="18">
@@ -1942,9 +1942,9 @@
         <v>81</v>
       </c>
     </row>
-    <row r="26" spans="1:9" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="23"/>
-      <c r="B26" s="25"/>
+    <row r="26" spans="1:9" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="46"/>
+      <c r="B26" s="48"/>
       <c r="C26" s="5">
         <v>23</v>
       </c>
@@ -1963,7 +1963,7 @@
       <c r="H26" s="5"/>
       <c r="I26" s="5"/>
     </row>
-    <row r="27" spans="1:9" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:9" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="6"/>
       <c r="B27" s="3"/>
       <c r="C27" s="4">
@@ -1972,15 +1972,15 @@
       <c r="D27" s="4">
         <v>8</v>
       </c>
-      <c r="E27" s="21" t="s">
+      <c r="E27" s="25" t="s">
         <v>31</v>
       </c>
-      <c r="F27" s="21"/>
-      <c r="G27" s="21"/>
-      <c r="H27" s="21"/>
-      <c r="I27" s="21"/>
-    </row>
-    <row r="28" spans="1:9" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="F27" s="25"/>
+      <c r="G27" s="25"/>
+      <c r="H27" s="25"/>
+      <c r="I27" s="25"/>
+    </row>
+    <row r="28" spans="1:9" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="6"/>
       <c r="B28" s="3"/>
       <c r="C28" s="4">
@@ -1989,19 +1989,19 @@
       <c r="D28" s="4">
         <v>9</v>
       </c>
-      <c r="E28" s="21" t="s">
+      <c r="E28" s="25" t="s">
         <v>31</v>
       </c>
-      <c r="F28" s="21"/>
-      <c r="G28" s="21"/>
-      <c r="H28" s="21"/>
-      <c r="I28" s="21"/>
-    </row>
-    <row r="29" spans="1:9" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="41" t="s">
+      <c r="F28" s="25"/>
+      <c r="G28" s="25"/>
+      <c r="H28" s="25"/>
+      <c r="I28" s="25"/>
+    </row>
+    <row r="29" spans="1:9" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="26" t="s">
         <v>95</v>
       </c>
-      <c r="B29" s="44" t="s">
+      <c r="B29" s="29" t="s">
         <v>97</v>
       </c>
       <c r="C29" s="17">
@@ -2024,9 +2024,9 @@
         <v>81</v>
       </c>
     </row>
-    <row r="30" spans="1:9" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="42"/>
-      <c r="B30" s="45"/>
+    <row r="30" spans="1:9" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="27"/>
+      <c r="B30" s="30"/>
       <c r="C30" s="1">
         <v>27</v>
       </c>
@@ -2045,9 +2045,9 @@
       <c r="H30" s="1"/>
       <c r="I30" s="1"/>
     </row>
-    <row r="31" spans="1:9" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="42"/>
-      <c r="B31" s="45"/>
+    <row r="31" spans="1:9" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="27"/>
+      <c r="B31" s="30"/>
       <c r="C31" s="17">
         <v>28</v>
       </c>
@@ -2066,9 +2066,9 @@
       <c r="H31" s="17"/>
       <c r="I31" s="17"/>
     </row>
-    <row r="32" spans="1:9" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="42"/>
-      <c r="B32" s="45"/>
+    <row r="32" spans="1:9" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="27"/>
+      <c r="B32" s="30"/>
       <c r="C32" s="1">
         <v>29</v>
       </c>
@@ -2087,9 +2087,9 @@
       <c r="H32" s="1"/>
       <c r="I32" s="1"/>
     </row>
-    <row r="33" spans="1:9" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A33" s="43"/>
-      <c r="B33" s="46"/>
+    <row r="33" spans="1:9" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="28"/>
+      <c r="B33" s="31"/>
       <c r="C33" s="17">
         <v>30</v>
       </c>
@@ -2108,11 +2108,11 @@
       <c r="H33" s="17"/>
       <c r="I33" s="17"/>
     </row>
-    <row r="34" spans="1:9" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="39" t="s">
+    <row r="34" spans="1:9" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="23" t="s">
         <v>62</v>
       </c>
-      <c r="B34" s="40" t="s">
+      <c r="B34" s="24" t="s">
         <v>83</v>
       </c>
       <c r="C34" s="2">
@@ -2135,9 +2135,9 @@
         <v>86</v>
       </c>
     </row>
-    <row r="35" spans="1:9" ht="14.15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="39"/>
-      <c r="B35" s="40"/>
+    <row r="35" spans="1:9" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="23"/>
+      <c r="B35" s="24"/>
       <c r="C35" s="12">
         <v>32</v>
       </c>
@@ -2160,11 +2160,13 @@
     </row>
   </sheetData>
   <mergeCells count="23">
-    <mergeCell ref="A34:A35"/>
-    <mergeCell ref="B34:B35"/>
-    <mergeCell ref="E28:I28"/>
-    <mergeCell ref="A29:A33"/>
-    <mergeCell ref="B29:B33"/>
+    <mergeCell ref="E27:I27"/>
+    <mergeCell ref="A25:A26"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="A20:A22"/>
+    <mergeCell ref="B20:B22"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="B23:B24"/>
     <mergeCell ref="B18:B19"/>
     <mergeCell ref="A1:B2"/>
     <mergeCell ref="G1:I2"/>
@@ -2176,13 +2178,11 @@
     <mergeCell ref="A4:A13"/>
     <mergeCell ref="B4:B13"/>
     <mergeCell ref="E17:I17"/>
-    <mergeCell ref="E27:I27"/>
-    <mergeCell ref="A25:A26"/>
-    <mergeCell ref="B25:B26"/>
-    <mergeCell ref="A20:A22"/>
-    <mergeCell ref="B20:B22"/>
-    <mergeCell ref="A23:A24"/>
-    <mergeCell ref="B23:B24"/>
+    <mergeCell ref="A34:A35"/>
+    <mergeCell ref="B34:B35"/>
+    <mergeCell ref="E28:I28"/>
+    <mergeCell ref="A29:A33"/>
+    <mergeCell ref="B29:B33"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2193,16 +2193,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{036672A4-8952-44C6-9E0D-0D4906E8D835}">
   <dimension ref="A1:P35"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="8" width="8.7265625" customWidth="1"/>
+    <col min="1" max="8" width="8.7109375" customWidth="1"/>
     <col min="9" max="10" width="2" customWidth="1"/>
-    <col min="11" max="12" width="7.26953125" customWidth="1"/>
-    <col min="13" max="13" width="7.26953125" hidden="1" customWidth="1"/>
-    <col min="14" max="14" width="7.26953125" customWidth="1"/>
+    <col min="11" max="12" width="7.28515625" customWidth="1"/>
+    <col min="13" max="13" width="7.28515625" hidden="1" customWidth="1"/>
+    <col min="14" max="14" width="7.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:16" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="33" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
@@ -2226,7 +2226,7 @@
       <c r="O1" s="35"/>
       <c r="P1" s="35"/>
     </row>
-    <row r="2" spans="1:16" ht="22" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:16" ht="21.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="34"/>
       <c r="B2" s="34"/>
       <c r="C2" s="37"/>
@@ -2244,51 +2244,51 @@
       <c r="O2" s="35"/>
       <c r="P2" s="35"/>
     </row>
-    <row r="3" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="55" t="s">
+    <row r="3" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="57" t="s">
         <v>103</v>
       </c>
-      <c r="B3" s="55"/>
-      <c r="C3" s="55"/>
-      <c r="D3" s="55"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="55"/>
-      <c r="G3" s="55"/>
-      <c r="H3" s="55"/>
+      <c r="B3" s="57"/>
+      <c r="C3" s="57"/>
+      <c r="D3" s="57"/>
+      <c r="E3" s="57"/>
+      <c r="F3" s="57"/>
+      <c r="G3" s="57"/>
+      <c r="H3" s="57"/>
       <c r="I3" s="11"/>
-      <c r="K3" s="47" t="s">
+      <c r="K3" s="74" t="s">
         <v>20</v>
       </c>
-      <c r="L3" s="47"/>
-      <c r="M3" s="47"/>
-      <c r="N3" s="47"/>
-      <c r="O3" s="47"/>
-      <c r="P3" s="47"/>
-    </row>
-    <row r="4" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="55" t="s">
+      <c r="L3" s="74"/>
+      <c r="M3" s="74"/>
+      <c r="N3" s="74"/>
+      <c r="O3" s="74"/>
+      <c r="P3" s="74"/>
+    </row>
+    <row r="4" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="57" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="55"/>
-      <c r="C4" s="55"/>
-      <c r="D4" s="55"/>
-      <c r="E4" s="55"/>
-      <c r="F4" s="55"/>
-      <c r="G4" s="55"/>
-      <c r="H4" s="55"/>
+      <c r="B4" s="57"/>
+      <c r="C4" s="57"/>
+      <c r="D4" s="57"/>
+      <c r="E4" s="57"/>
+      <c r="F4" s="57"/>
+      <c r="G4" s="57"/>
+      <c r="H4" s="57"/>
       <c r="I4" s="11"/>
-      <c r="K4" s="48">
+      <c r="K4" s="75">
         <v>1</v>
       </c>
-      <c r="L4" s="50" t="s">
+      <c r="L4" s="77" t="s">
         <v>68</v>
       </c>
-      <c r="M4" s="50"/>
-      <c r="N4" s="50"/>
-      <c r="O4" s="50"/>
-      <c r="P4" s="50"/>
-    </row>
-    <row r="5" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="M4" s="77"/>
+      <c r="N4" s="77"/>
+      <c r="O4" s="77"/>
+      <c r="P4" s="77"/>
+    </row>
+    <row r="5" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10">
         <v>1</v>
       </c>
@@ -2314,68 +2314,68 @@
         <v>8</v>
       </c>
       <c r="I5" s="11"/>
-      <c r="K5" s="49"/>
-      <c r="L5" s="50"/>
-      <c r="M5" s="50"/>
-      <c r="N5" s="50"/>
-      <c r="O5" s="50"/>
-      <c r="P5" s="50"/>
-    </row>
-    <row r="6" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="77" t="s">
+      <c r="K5" s="76"/>
+      <c r="L5" s="77"/>
+      <c r="M5" s="77"/>
+      <c r="N5" s="77"/>
+      <c r="O5" s="77"/>
+      <c r="P5" s="77"/>
+    </row>
+    <row r="6" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="58" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="77" t="s">
+      <c r="B6" s="58" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="77" t="s">
+      <c r="C6" s="58" t="s">
         <v>11</v>
       </c>
-      <c r="D6" s="77" t="s">
+      <c r="D6" s="58" t="s">
         <v>16</v>
       </c>
-      <c r="E6" s="77" t="s">
+      <c r="E6" s="58" t="s">
         <v>12</v>
       </c>
-      <c r="F6" s="77" t="s">
+      <c r="F6" s="58" t="s">
         <v>13</v>
       </c>
-      <c r="G6" s="77" t="s">
+      <c r="G6" s="58" t="s">
         <v>14</v>
       </c>
-      <c r="H6" s="78" t="s">
+      <c r="H6" s="71" t="s">
         <v>15</v>
       </c>
       <c r="I6" s="11"/>
-      <c r="K6" s="47">
+      <c r="K6" s="74">
         <v>2</v>
       </c>
-      <c r="L6" s="51" t="s">
+      <c r="L6" s="73" t="s">
         <v>69</v>
       </c>
-      <c r="M6" s="51"/>
-      <c r="N6" s="51"/>
-      <c r="O6" s="51"/>
-      <c r="P6" s="51"/>
-    </row>
-    <row r="7" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="77"/>
-      <c r="B7" s="77"/>
-      <c r="C7" s="77"/>
-      <c r="D7" s="77"/>
-      <c r="E7" s="77"/>
-      <c r="F7" s="77"/>
-      <c r="G7" s="77"/>
-      <c r="H7" s="79"/>
+      <c r="M6" s="73"/>
+      <c r="N6" s="73"/>
+      <c r="O6" s="73"/>
+      <c r="P6" s="73"/>
+    </row>
+    <row r="7" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="58"/>
+      <c r="B7" s="58"/>
+      <c r="C7" s="58"/>
+      <c r="D7" s="58"/>
+      <c r="E7" s="58"/>
+      <c r="F7" s="58"/>
+      <c r="G7" s="58"/>
+      <c r="H7" s="72"/>
       <c r="I7" s="11"/>
-      <c r="K7" s="47"/>
-      <c r="L7" s="51"/>
-      <c r="M7" s="51"/>
-      <c r="N7" s="51"/>
-      <c r="O7" s="51"/>
-      <c r="P7" s="51"/>
-    </row>
-    <row r="8" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="K7" s="74"/>
+      <c r="L7" s="73"/>
+      <c r="M7" s="73"/>
+      <c r="N7" s="73"/>
+      <c r="O7" s="73"/>
+      <c r="P7" s="73"/>
+    </row>
+    <row r="8" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="16"/>
       <c r="B8" s="16"/>
       <c r="C8" s="16"/>
@@ -2385,18 +2385,18 @@
       <c r="G8" s="16"/>
       <c r="H8" s="16"/>
       <c r="I8" s="11"/>
-      <c r="K8" s="48">
+      <c r="K8" s="75">
         <v>3</v>
       </c>
-      <c r="L8" s="50" t="s">
+      <c r="L8" s="77" t="s">
         <v>61</v>
       </c>
-      <c r="M8" s="50"/>
-      <c r="N8" s="50"/>
-      <c r="O8" s="50"/>
-      <c r="P8" s="50"/>
-    </row>
-    <row r="9" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="M8" s="77"/>
+      <c r="N8" s="77"/>
+      <c r="O8" s="77"/>
+      <c r="P8" s="77"/>
+    </row>
+    <row r="9" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="10">
         <v>9</v>
       </c>
@@ -2422,92 +2422,92 @@
         <v>16</v>
       </c>
       <c r="I9" s="11"/>
-      <c r="K9" s="49"/>
-      <c r="L9" s="50"/>
-      <c r="M9" s="50"/>
-      <c r="N9" s="50"/>
-      <c r="O9" s="50"/>
-      <c r="P9" s="50"/>
-    </row>
-    <row r="10" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="78" t="s">
+      <c r="K9" s="76"/>
+      <c r="L9" s="77"/>
+      <c r="M9" s="77"/>
+      <c r="N9" s="77"/>
+      <c r="O9" s="77"/>
+      <c r="P9" s="77"/>
+    </row>
+    <row r="10" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="71" t="s">
         <v>54</v>
       </c>
-      <c r="B10" s="77" t="s">
+      <c r="B10" s="58" t="s">
         <v>53</v>
       </c>
-      <c r="C10" s="54"/>
-      <c r="D10" s="54"/>
-      <c r="E10" s="54"/>
-      <c r="F10" s="54"/>
-      <c r="G10" s="58" t="s">
+      <c r="C10" s="64"/>
+      <c r="D10" s="64"/>
+      <c r="E10" s="64"/>
+      <c r="F10" s="64"/>
+      <c r="G10" s="67" t="s">
         <v>58</v>
       </c>
-      <c r="H10" s="58" t="s">
+      <c r="H10" s="67" t="s">
         <v>90</v>
       </c>
       <c r="I10" s="11"/>
-      <c r="K10" s="47">
+      <c r="K10" s="74">
         <v>4</v>
       </c>
-      <c r="L10" s="52" t="s">
+      <c r="L10" s="78" t="s">
         <v>70</v>
       </c>
-      <c r="M10" s="52"/>
-      <c r="N10" s="52"/>
-      <c r="O10" s="52"/>
-      <c r="P10" s="52"/>
-    </row>
-    <row r="11" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="79"/>
-      <c r="B11" s="77"/>
-      <c r="C11" s="54"/>
-      <c r="D11" s="54"/>
-      <c r="E11" s="54"/>
-      <c r="F11" s="54"/>
-      <c r="G11" s="58"/>
-      <c r="H11" s="58"/>
+      <c r="M10" s="78"/>
+      <c r="N10" s="78"/>
+      <c r="O10" s="78"/>
+      <c r="P10" s="78"/>
+    </row>
+    <row r="11" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="72"/>
+      <c r="B11" s="58"/>
+      <c r="C11" s="64"/>
+      <c r="D11" s="64"/>
+      <c r="E11" s="64"/>
+      <c r="F11" s="64"/>
+      <c r="G11" s="67"/>
+      <c r="H11" s="67"/>
       <c r="I11" s="11"/>
-      <c r="K11" s="47"/>
-      <c r="L11" s="52"/>
-      <c r="M11" s="52"/>
-      <c r="N11" s="52"/>
-      <c r="O11" s="52"/>
-      <c r="P11" s="52"/>
-    </row>
-    <row r="12" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="K11" s="74"/>
+      <c r="L11" s="78"/>
+      <c r="M11" s="78"/>
+      <c r="N11" s="78"/>
+      <c r="O11" s="78"/>
+      <c r="P11" s="78"/>
+    </row>
+    <row r="12" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I12" s="11"/>
-      <c r="K12" s="48">
+      <c r="K12" s="75">
         <v>5</v>
       </c>
-      <c r="L12" s="53" t="s">
+      <c r="L12" s="79" t="s">
         <v>101</v>
       </c>
-      <c r="M12" s="53"/>
-      <c r="N12" s="53"/>
-      <c r="O12" s="53"/>
-      <c r="P12" s="53"/>
-    </row>
-    <row r="13" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="55" t="s">
+      <c r="M12" s="79"/>
+      <c r="N12" s="79"/>
+      <c r="O12" s="79"/>
+      <c r="P12" s="79"/>
+    </row>
+    <row r="13" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="57" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="55"/>
-      <c r="C13" s="55"/>
-      <c r="D13" s="55"/>
-      <c r="E13" s="55"/>
-      <c r="F13" s="55"/>
-      <c r="G13" s="55"/>
-      <c r="H13" s="55"/>
+      <c r="B13" s="57"/>
+      <c r="C13" s="57"/>
+      <c r="D13" s="57"/>
+      <c r="E13" s="57"/>
+      <c r="F13" s="57"/>
+      <c r="G13" s="57"/>
+      <c r="H13" s="57"/>
       <c r="I13" s="11"/>
-      <c r="K13" s="49"/>
-      <c r="L13" s="53"/>
-      <c r="M13" s="53"/>
-      <c r="N13" s="53"/>
-      <c r="O13" s="53"/>
-      <c r="P13" s="53"/>
-    </row>
-    <row r="14" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="K13" s="76"/>
+      <c r="L13" s="79"/>
+      <c r="M13" s="79"/>
+      <c r="N13" s="79"/>
+      <c r="O13" s="79"/>
+      <c r="P13" s="79"/>
+    </row>
+    <row r="14" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="10">
         <v>1</v>
       </c>
@@ -2533,58 +2533,58 @@
         <v>8</v>
       </c>
       <c r="I14" s="11"/>
-      <c r="K14" s="47">
+      <c r="K14" s="74">
         <v>6</v>
       </c>
-      <c r="L14" s="51" t="s">
+      <c r="L14" s="73" t="s">
         <v>100</v>
       </c>
-      <c r="M14" s="51"/>
-      <c r="N14" s="51"/>
-      <c r="O14" s="51"/>
-      <c r="P14" s="51"/>
-    </row>
-    <row r="15" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="77" t="s">
+      <c r="M14" s="73"/>
+      <c r="N14" s="73"/>
+      <c r="O14" s="73"/>
+      <c r="P14" s="73"/>
+    </row>
+    <row r="15" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="58" t="s">
         <v>17</v>
       </c>
-      <c r="B15" s="77" t="s">
+      <c r="B15" s="58" t="s">
         <v>12</v>
       </c>
-      <c r="C15" s="77" t="s">
+      <c r="C15" s="58" t="s">
         <v>13</v>
       </c>
-      <c r="D15" s="77" t="s">
+      <c r="D15" s="58" t="s">
         <v>14</v>
       </c>
-      <c r="E15" s="77" t="s">
+      <c r="E15" s="58" t="s">
         <v>15</v>
       </c>
-      <c r="F15" s="77" t="s">
+      <c r="F15" s="58" t="s">
         <v>16</v>
       </c>
-      <c r="G15" s="54"/>
-      <c r="H15" s="54"/>
+      <c r="G15" s="64"/>
+      <c r="H15" s="64"/>
       <c r="I15" s="11"/>
-      <c r="K15" s="47"/>
-      <c r="L15" s="51"/>
-      <c r="M15" s="51"/>
-      <c r="N15" s="51"/>
-      <c r="O15" s="51"/>
-      <c r="P15" s="51"/>
-    </row>
-    <row r="16" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A16" s="77"/>
-      <c r="B16" s="77"/>
-      <c r="C16" s="77"/>
-      <c r="D16" s="77"/>
-      <c r="E16" s="77"/>
-      <c r="F16" s="77"/>
-      <c r="G16" s="54"/>
-      <c r="H16" s="54"/>
+      <c r="K15" s="74"/>
+      <c r="L15" s="73"/>
+      <c r="M15" s="73"/>
+      <c r="N15" s="73"/>
+      <c r="O15" s="73"/>
+      <c r="P15" s="73"/>
+    </row>
+    <row r="16" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="58"/>
+      <c r="B16" s="58"/>
+      <c r="C16" s="58"/>
+      <c r="D16" s="58"/>
+      <c r="E16" s="58"/>
+      <c r="F16" s="58"/>
+      <c r="G16" s="64"/>
+      <c r="H16" s="64"/>
       <c r="I16" s="11"/>
     </row>
-    <row r="17" spans="1:9" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:9" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="19"/>
       <c r="B17" s="19"/>
       <c r="C17" s="19"/>
@@ -2595,36 +2595,36 @@
       <c r="H17" s="19"/>
       <c r="I17" s="20"/>
     </row>
-    <row r="18" spans="1:9" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:9" ht="15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="I18" s="11"/>
     </row>
-    <row r="19" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="55" t="s">
+    <row r="19" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="57" t="s">
         <v>104</v>
       </c>
-      <c r="B19" s="55"/>
-      <c r="C19" s="55"/>
-      <c r="D19" s="55"/>
-      <c r="E19" s="55"/>
-      <c r="F19" s="55"/>
-      <c r="G19" s="55"/>
-      <c r="H19" s="55"/>
+      <c r="B19" s="57"/>
+      <c r="C19" s="57"/>
+      <c r="D19" s="57"/>
+      <c r="E19" s="57"/>
+      <c r="F19" s="57"/>
+      <c r="G19" s="57"/>
+      <c r="H19" s="57"/>
       <c r="I19" s="11"/>
     </row>
-    <row r="20" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A20" s="55" t="s">
+    <row r="20" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="57" t="s">
         <v>0</v>
       </c>
-      <c r="B20" s="55"/>
-      <c r="C20" s="55"/>
-      <c r="D20" s="55"/>
-      <c r="E20" s="55"/>
-      <c r="F20" s="55"/>
-      <c r="G20" s="55"/>
-      <c r="H20" s="55"/>
+      <c r="B20" s="57"/>
+      <c r="C20" s="57"/>
+      <c r="D20" s="57"/>
+      <c r="E20" s="57"/>
+      <c r="F20" s="57"/>
+      <c r="G20" s="57"/>
+      <c r="H20" s="57"/>
       <c r="I20" s="11"/>
     </row>
-    <row r="21" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="10">
         <v>1</v>
       </c>
@@ -2651,43 +2651,43 @@
       </c>
       <c r="I21" s="11"/>
     </row>
-    <row r="22" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="67" t="s">
+    <row r="22" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="55" t="s">
         <v>18</v>
       </c>
-      <c r="B22" s="56" t="s">
+      <c r="B22" s="60" t="s">
         <v>19</v>
       </c>
-      <c r="C22" s="56" t="s">
+      <c r="C22" s="60" t="s">
         <v>56</v>
       </c>
-      <c r="D22" s="57" t="s">
+      <c r="D22" s="61" t="s">
         <v>47</v>
       </c>
-      <c r="E22" s="57" t="s">
+      <c r="E22" s="61" t="s">
         <v>64</v>
       </c>
-      <c r="F22" s="63" t="s">
+      <c r="F22" s="68" t="s">
         <v>1</v>
       </c>
-      <c r="G22" s="63" t="s">
+      <c r="G22" s="68" t="s">
         <v>2</v>
       </c>
-      <c r="H22" s="54"/>
+      <c r="H22" s="64"/>
       <c r="I22" s="11"/>
     </row>
-    <row r="23" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="68"/>
-      <c r="B23" s="56"/>
-      <c r="C23" s="56"/>
-      <c r="D23" s="57"/>
-      <c r="E23" s="57"/>
-      <c r="F23" s="63"/>
-      <c r="G23" s="63"/>
-      <c r="H23" s="54"/>
+    <row r="23" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="56"/>
+      <c r="B23" s="60"/>
+      <c r="C23" s="60"/>
+      <c r="D23" s="61"/>
+      <c r="E23" s="61"/>
+      <c r="F23" s="68"/>
+      <c r="G23" s="68"/>
+      <c r="H23" s="64"/>
       <c r="I23" s="11"/>
     </row>
-    <row r="24" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="16"/>
       <c r="B24" s="16"/>
       <c r="C24" s="16"/>
@@ -2698,7 +2698,7 @@
       <c r="H24" s="16"/>
       <c r="I24" s="11"/>
     </row>
-    <row r="25" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="10">
         <v>9</v>
       </c>
@@ -2725,59 +2725,59 @@
       </c>
       <c r="I25" s="11"/>
     </row>
-    <row r="26" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A26" s="59"/>
-      <c r="B26" s="61" t="s">
+    <row r="26" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="69"/>
+      <c r="B26" s="65" t="s">
         <v>3</v>
       </c>
-      <c r="C26" s="61" t="s">
+      <c r="C26" s="65" t="s">
         <v>4</v>
       </c>
-      <c r="D26" s="61" t="s">
+      <c r="D26" s="65" t="s">
         <v>5</v>
       </c>
-      <c r="E26" s="61" t="s">
+      <c r="E26" s="65" t="s">
         <v>6</v>
       </c>
-      <c r="F26" s="61" t="s">
+      <c r="F26" s="65" t="s">
         <v>7</v>
       </c>
-      <c r="G26" s="58" t="s">
+      <c r="G26" s="67" t="s">
         <v>84</v>
       </c>
-      <c r="H26" s="58" t="s">
+      <c r="H26" s="67" t="s">
         <v>85</v>
       </c>
       <c r="I26" s="11"/>
     </row>
-    <row r="27" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A27" s="60"/>
-      <c r="B27" s="62"/>
-      <c r="C27" s="62"/>
-      <c r="D27" s="62"/>
-      <c r="E27" s="62"/>
-      <c r="F27" s="62"/>
-      <c r="G27" s="58"/>
-      <c r="H27" s="58"/>
+    <row r="27" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="70"/>
+      <c r="B27" s="66"/>
+      <c r="C27" s="66"/>
+      <c r="D27" s="66"/>
+      <c r="E27" s="66"/>
+      <c r="F27" s="66"/>
+      <c r="G27" s="67"/>
+      <c r="H27" s="67"/>
       <c r="I27" s="11"/>
     </row>
-    <row r="28" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I28" s="11"/>
     </row>
-    <row r="29" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="55" t="s">
+    <row r="29" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="57" t="s">
         <v>8</v>
       </c>
-      <c r="B29" s="55"/>
-      <c r="C29" s="55"/>
-      <c r="D29" s="55"/>
-      <c r="E29" s="55"/>
-      <c r="F29" s="55"/>
-      <c r="G29" s="55"/>
-      <c r="H29" s="55"/>
+      <c r="B29" s="57"/>
+      <c r="C29" s="57"/>
+      <c r="D29" s="57"/>
+      <c r="E29" s="57"/>
+      <c r="F29" s="57"/>
+      <c r="G29" s="57"/>
+      <c r="H29" s="57"/>
       <c r="I29" s="11"/>
     </row>
-    <row r="30" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="10">
         <v>1</v>
       </c>
@@ -2804,77 +2804,75 @@
       </c>
       <c r="I30" s="11"/>
     </row>
-    <row r="31" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="77" t="s">
+    <row r="31" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="58" t="s">
         <v>72</v>
       </c>
-      <c r="B31" s="56" t="s">
+      <c r="B31" s="60" t="s">
         <v>75</v>
       </c>
-      <c r="C31" s="57" t="s">
+      <c r="C31" s="61" t="s">
         <v>74</v>
       </c>
-      <c r="D31" s="65" t="s">
+      <c r="D31" s="62" t="s">
         <v>71</v>
       </c>
-      <c r="E31" s="66" t="s">
+      <c r="E31" s="63" t="s">
         <v>73</v>
       </c>
-      <c r="F31" s="54"/>
-      <c r="G31" s="64" t="s">
+      <c r="F31" s="64"/>
+      <c r="G31" s="59" t="s">
         <v>9</v>
       </c>
-      <c r="H31" s="64" t="s">
+      <c r="H31" s="59" t="s">
         <v>66</v>
       </c>
       <c r="I31" s="11"/>
     </row>
-    <row r="32" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="77"/>
-      <c r="B32" s="56"/>
-      <c r="C32" s="57"/>
-      <c r="D32" s="65"/>
-      <c r="E32" s="66"/>
-      <c r="F32" s="54"/>
-      <c r="G32" s="64"/>
-      <c r="H32" s="64"/>
+    <row r="32" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="58"/>
+      <c r="B32" s="60"/>
+      <c r="C32" s="61"/>
+      <c r="D32" s="62"/>
+      <c r="E32" s="63"/>
+      <c r="F32" s="64"/>
+      <c r="G32" s="59"/>
+      <c r="H32" s="59"/>
       <c r="I32" s="11"/>
     </row>
-    <row r="33" spans="9:9" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="9:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I33" s="11"/>
     </row>
-    <row r="34" spans="9:9" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
-    <row r="35" spans="9:9" ht="15" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="34" spans="9:9" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="35" spans="9:9" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="70">
-    <mergeCell ref="A22:A23"/>
-    <mergeCell ref="A19:H19"/>
-    <mergeCell ref="A20:H20"/>
-    <mergeCell ref="A15:A16"/>
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="C15:C16"/>
-    <mergeCell ref="D15:D16"/>
-    <mergeCell ref="E15:E16"/>
-    <mergeCell ref="A29:H29"/>
-    <mergeCell ref="G31:G32"/>
-    <mergeCell ref="H31:H32"/>
-    <mergeCell ref="A31:A32"/>
-    <mergeCell ref="B31:B32"/>
-    <mergeCell ref="C31:C32"/>
-    <mergeCell ref="D31:D32"/>
-    <mergeCell ref="E31:E32"/>
-    <mergeCell ref="F31:F32"/>
-    <mergeCell ref="F26:F27"/>
-    <mergeCell ref="G26:G27"/>
-    <mergeCell ref="H26:H27"/>
-    <mergeCell ref="F22:F23"/>
-    <mergeCell ref="G22:G23"/>
-    <mergeCell ref="H22:H23"/>
-    <mergeCell ref="A26:A27"/>
-    <mergeCell ref="B26:B27"/>
-    <mergeCell ref="C26:C27"/>
-    <mergeCell ref="D26:D27"/>
-    <mergeCell ref="E26:E27"/>
+    <mergeCell ref="K3:P3"/>
+    <mergeCell ref="K6:K7"/>
+    <mergeCell ref="K8:K9"/>
+    <mergeCell ref="K10:K11"/>
+    <mergeCell ref="K12:K13"/>
+    <mergeCell ref="K4:K5"/>
+    <mergeCell ref="L4:P5"/>
+    <mergeCell ref="L6:P7"/>
+    <mergeCell ref="L8:P9"/>
+    <mergeCell ref="L10:P11"/>
+    <mergeCell ref="L12:P13"/>
+    <mergeCell ref="L14:P15"/>
+    <mergeCell ref="K14:K15"/>
+    <mergeCell ref="C10:C11"/>
+    <mergeCell ref="D10:D11"/>
+    <mergeCell ref="E10:E11"/>
+    <mergeCell ref="G15:G16"/>
+    <mergeCell ref="H15:H16"/>
+    <mergeCell ref="A3:H3"/>
+    <mergeCell ref="A4:H4"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="C6:C7"/>
+    <mergeCell ref="D6:D7"/>
+    <mergeCell ref="E6:E7"/>
+    <mergeCell ref="F6:F7"/>
     <mergeCell ref="K1:P2"/>
     <mergeCell ref="B22:B23"/>
     <mergeCell ref="C22:C23"/>
@@ -2891,32 +2889,34 @@
     <mergeCell ref="F10:F11"/>
     <mergeCell ref="A13:H13"/>
     <mergeCell ref="F15:F16"/>
-    <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A4:H4"/>
-    <mergeCell ref="A6:A7"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="C6:C7"/>
-    <mergeCell ref="D6:D7"/>
-    <mergeCell ref="E6:E7"/>
-    <mergeCell ref="F6:F7"/>
-    <mergeCell ref="L14:P15"/>
-    <mergeCell ref="K14:K15"/>
-    <mergeCell ref="C10:C11"/>
-    <mergeCell ref="D10:D11"/>
-    <mergeCell ref="E10:E11"/>
-    <mergeCell ref="G15:G16"/>
-    <mergeCell ref="H15:H16"/>
-    <mergeCell ref="K3:P3"/>
-    <mergeCell ref="K6:K7"/>
-    <mergeCell ref="K8:K9"/>
-    <mergeCell ref="K10:K11"/>
-    <mergeCell ref="K12:K13"/>
-    <mergeCell ref="K4:K5"/>
-    <mergeCell ref="L4:P5"/>
-    <mergeCell ref="L6:P7"/>
-    <mergeCell ref="L8:P9"/>
-    <mergeCell ref="L10:P11"/>
-    <mergeCell ref="L12:P13"/>
+    <mergeCell ref="A26:A27"/>
+    <mergeCell ref="B26:B27"/>
+    <mergeCell ref="C26:C27"/>
+    <mergeCell ref="D26:D27"/>
+    <mergeCell ref="E26:E27"/>
+    <mergeCell ref="F26:F27"/>
+    <mergeCell ref="G26:G27"/>
+    <mergeCell ref="H26:H27"/>
+    <mergeCell ref="F22:F23"/>
+    <mergeCell ref="G22:G23"/>
+    <mergeCell ref="H22:H23"/>
+    <mergeCell ref="A29:H29"/>
+    <mergeCell ref="G31:G32"/>
+    <mergeCell ref="H31:H32"/>
+    <mergeCell ref="A31:A32"/>
+    <mergeCell ref="B31:B32"/>
+    <mergeCell ref="C31:C32"/>
+    <mergeCell ref="D31:D32"/>
+    <mergeCell ref="E31:E32"/>
+    <mergeCell ref="F31:F32"/>
+    <mergeCell ref="A22:A23"/>
+    <mergeCell ref="A19:H19"/>
+    <mergeCell ref="A20:H20"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="C15:C16"/>
+    <mergeCell ref="D15:D16"/>
+    <mergeCell ref="E15:E16"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Update Input List.xlsx with new data
</commit_message>
<xml_diff>
--- a/Input List/Full Band/Input List.xlsx
+++ b/Input List/Full Band/Input List.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="X:\TechnicalDocumentation\Input List\Full Band\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B6859FD-38EA-4A84-BD4E-9E5E280992B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB43103C-1B28-4CBF-BCC0-5200F71DA054}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{976BA9A3-41FE-45E5-BC0B-B40312D9AF21}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{976BA9A3-41FE-45E5-BC0B-B40312D9AF21}"/>
   </bookViews>
   <sheets>
     <sheet name="Channels" sheetId="1" r:id="rId1"/>
@@ -49,9 +49,10 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata">
-  <metadataTypes count="1">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="2">
     <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
   <futureMetadata name="XLRICHVALUE" count="1">
     <bk>
@@ -62,6 +63,20 @@
       </extLst>
     </bk>
   </futureMetadata>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="2" v="0"/>
+    </bk>
+  </cellMetadata>
   <valueMetadata count="1">
     <bk>
       <rc t="1" v="0"/>
@@ -548,7 +563,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="22" x14ac:knownFonts="1">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -674,14 +689,6 @@
     <font>
       <b/>
       <sz val="10"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="28"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -817,7 +824,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="14">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -963,20 +970,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="102">
+  <cellXfs count="106">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -997,14 +995,100 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1012,6 +1096,12 @@
     <xf numFmtId="0" fontId="6" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
@@ -1028,15 +1118,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
@@ -1053,6 +1134,9 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
@@ -1062,9 +1146,84 @@
     <xf numFmtId="0" fontId="13" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1107,169 +1266,20 @@
     <xf numFmtId="0" fontId="3" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="16" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="16" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="14" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="16" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="12" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="12" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="13" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="14" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1367,8 +1377,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1F06299C-206A-4E5B-812B-2628B9127415}" name="Table1" displayName="Table1" ref="K19:M24" totalsRowShown="0">
-  <autoFilter ref="K19:M24" xr:uid="{1F06299C-206A-4E5B-812B-2628B9127415}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1F06299C-206A-4E5B-812B-2628B9127415}" name="Table1" displayName="Table1" ref="K30:M35" totalsRowShown="0">
+  <autoFilter ref="K30:M35" xr:uid="{1F06299C-206A-4E5B-812B-2628B9127415}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{DBD1845E-C8E6-4D25-AB4B-500331BD2BF7}" name="Device"/>
     <tableColumn id="2" xr3:uid="{25C87226-CD3A-436C-AE3E-D8E60BFFEA83}" name="Model"/>
@@ -1690,844 +1700,849 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="24" t="e" vm="1">
+      <c r="A1" s="53" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="26" t="s">
+      <c r="B1" s="53"/>
+      <c r="C1" s="104" t="s">
         <v>109</v>
       </c>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
-      <c r="G1" s="26"/>
+      <c r="D1" s="104"/>
+      <c r="E1" s="104"/>
+      <c r="F1" s="55" t="str" cm="1">
+        <f t="array" aca="1" ref="F1" ca="1">" (" &amp; _xlfn.TEXTAFTER(CELL("filename", A1), "]") &amp; ")"</f>
+        <v xml:space="preserve"> (Channels)</v>
+      </c>
+      <c r="G1" s="55"/>
       <c r="H1" s="8" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="25"/>
-      <c r="B2" s="25"/>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27"/>
-      <c r="F2" s="27"/>
-      <c r="G2" s="27"/>
+      <c r="A2" s="54"/>
+      <c r="B2" s="54"/>
+      <c r="C2" s="105"/>
+      <c r="D2" s="105"/>
+      <c r="E2" s="105"/>
+      <c r="F2" s="56"/>
+      <c r="G2" s="56"/>
       <c r="H2" s="9" t="str">
         <f ca="1">"Date Updated: "&amp;TEXT(TODAY(),"yyyy.mm.dd")</f>
-        <v>Date Updated: 2026.01.02</v>
+        <v>Date Updated: 2026.01.03</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="66" t="s">
+      <c r="A3" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="B3" s="66" t="s">
+      <c r="B3" s="13" t="s">
         <v>62</v>
       </c>
-      <c r="C3" s="75" t="s">
+      <c r="C3" s="16" t="s">
         <v>144</v>
       </c>
-      <c r="D3" s="76" t="s">
+      <c r="D3" s="17" t="s">
         <v>68</v>
       </c>
-      <c r="E3" s="76" t="s">
+      <c r="E3" s="17" t="s">
         <v>147</v>
       </c>
-      <c r="F3" s="76" t="s">
+      <c r="F3" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="G3" s="76" t="s">
+      <c r="G3" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="H3" s="76" t="s">
+      <c r="H3" s="17" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="28" t="s">
+      <c r="A4" s="58" t="s">
         <v>42</v>
       </c>
-      <c r="B4" s="69" t="s">
+      <c r="B4" s="61" t="s">
         <v>24</v>
       </c>
-      <c r="C4" s="77">
+      <c r="C4" s="18">
         <v>1</v>
       </c>
-      <c r="D4" s="78" t="s">
+      <c r="D4" s="19" t="s">
         <v>73</v>
       </c>
-      <c r="E4" s="78" t="s">
+      <c r="E4" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="F4" s="78" t="s">
+      <c r="F4" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="G4" s="78" t="s">
+      <c r="G4" s="19" t="s">
         <v>69</v>
       </c>
-      <c r="H4" s="78" t="s">
+      <c r="H4" s="19" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="29"/>
-      <c r="B5" s="70"/>
-      <c r="C5" s="79">
+      <c r="A5" s="59"/>
+      <c r="B5" s="62"/>
+      <c r="C5" s="20">
         <v>2</v>
       </c>
-      <c r="D5" s="80" t="s">
+      <c r="D5" s="21" t="s">
         <v>74</v>
       </c>
-      <c r="E5" s="80" t="s">
+      <c r="E5" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="F5" s="80" t="s">
+      <c r="F5" s="21" t="s">
         <v>19</v>
       </c>
-      <c r="G5" s="80" t="s">
+      <c r="G5" s="21" t="s">
         <v>22</v>
       </c>
-      <c r="H5" s="80" t="s">
+      <c r="H5" s="21" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="29"/>
-      <c r="B6" s="70"/>
-      <c r="C6" s="77">
+      <c r="A6" s="59"/>
+      <c r="B6" s="62"/>
+      <c r="C6" s="18">
         <v>3</v>
       </c>
-      <c r="D6" s="78" t="s">
+      <c r="D6" s="19" t="s">
         <v>75</v>
       </c>
-      <c r="E6" s="78" t="s">
+      <c r="E6" s="19" t="s">
         <v>9</v>
       </c>
-      <c r="F6" s="78" t="s">
+      <c r="F6" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="G6" s="78" t="s">
+      <c r="G6" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="H6" s="78"/>
+      <c r="H6" s="19"/>
     </row>
     <row r="7" spans="1:8" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="29"/>
-      <c r="B7" s="70"/>
-      <c r="C7" s="79">
+      <c r="A7" s="59"/>
+      <c r="B7" s="62"/>
+      <c r="C7" s="20">
         <v>4</v>
       </c>
-      <c r="D7" s="80" t="s">
+      <c r="D7" s="21" t="s">
         <v>76</v>
       </c>
-      <c r="E7" s="80" t="s">
+      <c r="E7" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="F7" s="80" t="s">
+      <c r="F7" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="G7" s="80" t="s">
+      <c r="G7" s="21" t="s">
         <v>56</v>
       </c>
-      <c r="H7" s="80" t="s">
+      <c r="H7" s="21" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="29"/>
-      <c r="B8" s="70"/>
-      <c r="C8" s="77">
+      <c r="A8" s="59"/>
+      <c r="B8" s="62"/>
+      <c r="C8" s="18">
         <v>5</v>
       </c>
-      <c r="D8" s="78" t="s">
+      <c r="D8" s="19" t="s">
         <v>77</v>
       </c>
-      <c r="E8" s="78" t="s">
+      <c r="E8" s="19" t="s">
         <v>10</v>
       </c>
-      <c r="F8" s="78" t="s">
+      <c r="F8" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="G8" s="78" t="s">
+      <c r="G8" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="H8" s="78" t="s">
+      <c r="H8" s="19" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="29"/>
-      <c r="B9" s="70"/>
-      <c r="C9" s="79">
+      <c r="A9" s="59"/>
+      <c r="B9" s="62"/>
+      <c r="C9" s="20">
         <v>6</v>
       </c>
-      <c r="D9" s="80" t="s">
+      <c r="D9" s="21" t="s">
         <v>78</v>
       </c>
-      <c r="E9" s="80" t="s">
+      <c r="E9" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="F9" s="80" t="s">
+      <c r="F9" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="G9" s="80" t="s">
+      <c r="G9" s="21" t="s">
         <v>56</v>
       </c>
-      <c r="H9" s="80" t="s">
+      <c r="H9" s="21" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="29"/>
-      <c r="B10" s="70"/>
-      <c r="C10" s="77">
+      <c r="A10" s="59"/>
+      <c r="B10" s="62"/>
+      <c r="C10" s="18">
         <v>7</v>
       </c>
-      <c r="D10" s="78" t="s">
+      <c r="D10" s="19" t="s">
         <v>79</v>
       </c>
-      <c r="E10" s="78" t="s">
+      <c r="E10" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="F10" s="78" t="s">
+      <c r="F10" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="G10" s="78" t="s">
+      <c r="G10" s="19" t="s">
         <v>56</v>
       </c>
-      <c r="H10" s="78" t="s">
+      <c r="H10" s="19" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="29"/>
-      <c r="B11" s="70"/>
-      <c r="C11" s="79">
+      <c r="A11" s="59"/>
+      <c r="B11" s="62"/>
+      <c r="C11" s="20">
         <v>8</v>
       </c>
-      <c r="D11" s="80" t="s">
+      <c r="D11" s="21" t="s">
         <v>80</v>
       </c>
-      <c r="E11" s="80" t="s">
+      <c r="E11" s="21" t="s">
         <v>13</v>
       </c>
-      <c r="F11" s="80" t="s">
+      <c r="F11" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="G11" s="80" t="s">
+      <c r="G11" s="21" t="s">
         <v>56</v>
       </c>
-      <c r="H11" s="80" t="s">
+      <c r="H11" s="21" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="29"/>
-      <c r="B12" s="70"/>
-      <c r="C12" s="77">
+      <c r="A12" s="59"/>
+      <c r="B12" s="62"/>
+      <c r="C12" s="18">
         <v>9</v>
       </c>
-      <c r="D12" s="78" t="s">
+      <c r="D12" s="19" t="s">
         <v>81</v>
       </c>
-      <c r="E12" s="78" t="s">
+      <c r="E12" s="19" t="s">
         <v>44</v>
       </c>
-      <c r="F12" s="78" t="s">
+      <c r="F12" s="19" t="s">
         <v>23</v>
       </c>
-      <c r="G12" s="78" t="s">
+      <c r="G12" s="19" t="s">
         <v>70</v>
       </c>
-      <c r="H12" s="78" t="s">
+      <c r="H12" s="19" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="30"/>
-      <c r="B13" s="71"/>
-      <c r="C13" s="79">
+      <c r="A13" s="60"/>
+      <c r="B13" s="63"/>
+      <c r="C13" s="20">
         <v>10</v>
       </c>
-      <c r="D13" s="80" t="s">
+      <c r="D13" s="21" t="s">
         <v>82</v>
       </c>
-      <c r="E13" s="80" t="s">
+      <c r="E13" s="21" t="s">
         <v>43</v>
       </c>
-      <c r="F13" s="80" t="s">
+      <c r="F13" s="21" t="s">
         <v>23</v>
       </c>
-      <c r="G13" s="80" t="s">
+      <c r="G13" s="21" t="s">
         <v>70</v>
       </c>
-      <c r="H13" s="80" t="s">
+      <c r="H13" s="21" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3"/>
       <c r="B14" s="3"/>
-      <c r="C14" s="81">
+      <c r="C14" s="22">
         <v>11</v>
       </c>
-      <c r="D14" s="82"/>
-      <c r="E14" s="67" t="s">
+      <c r="D14" s="23"/>
+      <c r="E14" s="57" t="s">
         <v>25</v>
       </c>
-      <c r="F14" s="67"/>
-      <c r="G14" s="67"/>
-      <c r="H14" s="67"/>
+      <c r="F14" s="57"/>
+      <c r="G14" s="57"/>
+      <c r="H14" s="57"/>
     </row>
     <row r="15" spans="1:8" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3"/>
       <c r="B15" s="3"/>
-      <c r="C15" s="81">
+      <c r="C15" s="22">
         <v>12</v>
       </c>
-      <c r="D15" s="82"/>
-      <c r="E15" s="67" t="s">
+      <c r="D15" s="23"/>
+      <c r="E15" s="57" t="s">
         <v>25</v>
       </c>
-      <c r="F15" s="67"/>
-      <c r="G15" s="67"/>
-      <c r="H15" s="67"/>
+      <c r="F15" s="57"/>
+      <c r="G15" s="57"/>
+      <c r="H15" s="57"/>
     </row>
     <row r="16" spans="1:8" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3"/>
       <c r="B16" s="3"/>
-      <c r="C16" s="81">
+      <c r="C16" s="22">
         <v>13</v>
       </c>
-      <c r="D16" s="82"/>
-      <c r="E16" s="67" t="s">
+      <c r="D16" s="23"/>
+      <c r="E16" s="57" t="s">
         <v>25</v>
       </c>
-      <c r="F16" s="67"/>
-      <c r="G16" s="67"/>
-      <c r="H16" s="67"/>
+      <c r="F16" s="57"/>
+      <c r="G16" s="57"/>
+      <c r="H16" s="57"/>
     </row>
     <row r="17" spans="1:8" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="13" t="s">
+      <c r="A17" s="43" t="s">
         <v>115</v>
       </c>
-      <c r="B17" s="72" t="s">
+      <c r="B17" s="45" t="s">
         <v>92</v>
       </c>
-      <c r="C17" s="83">
+      <c r="C17" s="24">
         <v>14</v>
       </c>
-      <c r="D17" s="84" t="s">
+      <c r="D17" s="25" t="s">
         <v>83</v>
       </c>
-      <c r="E17" s="84" t="s">
+      <c r="E17" s="25" t="s">
         <v>117</v>
       </c>
-      <c r="F17" s="84" t="s">
+      <c r="F17" s="25" t="s">
         <v>26</v>
       </c>
-      <c r="G17" s="84" t="s">
+      <c r="G17" s="25" t="s">
         <v>70</v>
       </c>
-      <c r="H17" s="84" t="s">
+      <c r="H17" s="25" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="14"/>
-      <c r="B18" s="73"/>
-      <c r="C18" s="85">
+      <c r="A18" s="44"/>
+      <c r="B18" s="46"/>
+      <c r="C18" s="26">
         <v>15</v>
       </c>
-      <c r="D18" s="86" t="s">
+      <c r="D18" s="27" t="s">
         <v>84</v>
       </c>
-      <c r="E18" s="86" t="s">
+      <c r="E18" s="27" t="s">
         <v>118</v>
       </c>
-      <c r="F18" s="86" t="s">
+      <c r="F18" s="27" t="s">
         <v>28</v>
       </c>
-      <c r="G18" s="86" t="s">
+      <c r="G18" s="27" t="s">
         <v>29</v>
       </c>
-      <c r="H18" s="86"/>
+      <c r="H18" s="27"/>
     </row>
     <row r="19" spans="1:8" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="46"/>
-      <c r="B19" s="46"/>
-      <c r="C19" s="81">
+      <c r="A19" s="10"/>
+      <c r="B19" s="10"/>
+      <c r="C19" s="22">
         <v>16</v>
       </c>
-      <c r="D19" s="87"/>
-      <c r="E19" s="67" t="s">
+      <c r="D19" s="28"/>
+      <c r="E19" s="57" t="s">
         <v>25</v>
       </c>
-      <c r="F19" s="67"/>
-      <c r="G19" s="67"/>
-      <c r="H19" s="67"/>
+      <c r="F19" s="57"/>
+      <c r="G19" s="57"/>
+      <c r="H19" s="57"/>
     </row>
     <row r="20" spans="1:8" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="23" t="s">
+      <c r="A20" s="64" t="s">
         <v>63</v>
       </c>
-      <c r="B20" s="23" t="s">
+      <c r="B20" s="64" t="s">
         <v>66</v>
       </c>
-      <c r="C20" s="88">
+      <c r="C20" s="29">
         <v>17</v>
       </c>
-      <c r="D20" s="89" t="s">
+      <c r="D20" s="30" t="s">
         <v>85</v>
       </c>
-      <c r="E20" s="89" t="s">
+      <c r="E20" s="30" t="s">
         <v>39</v>
       </c>
-      <c r="F20" s="89" t="s">
+      <c r="F20" s="30" t="s">
         <v>40</v>
       </c>
-      <c r="G20" s="89" t="s">
+      <c r="G20" s="30" t="s">
         <v>70</v>
       </c>
-      <c r="H20" s="89" t="s">
+      <c r="H20" s="30" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="21" spans="1:8" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="23"/>
-      <c r="B21" s="23"/>
-      <c r="C21" s="90">
+      <c r="A21" s="64"/>
+      <c r="B21" s="64"/>
+      <c r="C21" s="31">
         <v>18</v>
       </c>
-      <c r="D21" s="91" t="s">
+      <c r="D21" s="32" t="s">
         <v>113</v>
       </c>
-      <c r="E21" s="91" t="s">
+      <c r="E21" s="32" t="s">
         <v>47</v>
       </c>
-      <c r="F21" s="91" t="s">
+      <c r="F21" s="32" t="s">
         <v>48</v>
       </c>
-      <c r="G21" s="91" t="s">
+      <c r="G21" s="32" t="s">
         <v>29</v>
       </c>
-      <c r="H21" s="91"/>
+      <c r="H21" s="32"/>
     </row>
     <row r="22" spans="1:8" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="74"/>
-      <c r="B22" s="74"/>
-      <c r="C22" s="81">
+      <c r="A22" s="15"/>
+      <c r="B22" s="15"/>
+      <c r="C22" s="22">
         <v>19</v>
       </c>
-      <c r="D22" s="87"/>
-      <c r="E22" s="67" t="s">
+      <c r="D22" s="28"/>
+      <c r="E22" s="57" t="s">
         <v>25</v>
       </c>
-      <c r="F22" s="67"/>
-      <c r="G22" s="67"/>
-      <c r="H22" s="67"/>
+      <c r="F22" s="57"/>
+      <c r="G22" s="57"/>
+      <c r="H22" s="57"/>
     </row>
     <row r="23" spans="1:8" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="10" t="s">
+      <c r="A23" s="65" t="s">
         <v>64</v>
       </c>
-      <c r="B23" s="10" t="s">
+      <c r="B23" s="65" t="s">
         <v>67</v>
       </c>
-      <c r="C23" s="92">
+      <c r="C23" s="33">
         <v>20</v>
       </c>
-      <c r="D23" s="93" t="s">
+      <c r="D23" s="34" t="s">
         <v>96</v>
       </c>
-      <c r="E23" s="93" t="s">
+      <c r="E23" s="34" t="s">
         <v>1</v>
       </c>
-      <c r="F23" s="93" t="s">
+      <c r="F23" s="34" t="s">
         <v>32</v>
       </c>
-      <c r="G23" s="93" t="s">
+      <c r="G23" s="34" t="s">
         <v>70</v>
       </c>
-      <c r="H23" s="93" t="s">
+      <c r="H23" s="34" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="11"/>
-      <c r="B24" s="11"/>
-      <c r="C24" s="94">
+      <c r="A24" s="66"/>
+      <c r="B24" s="66"/>
+      <c r="C24" s="35">
         <v>21</v>
       </c>
-      <c r="D24" s="95" t="s">
+      <c r="D24" s="36" t="s">
         <v>110</v>
       </c>
-      <c r="E24" s="95" t="s">
+      <c r="E24" s="36" t="s">
         <v>2</v>
       </c>
-      <c r="F24" s="95" t="s">
+      <c r="F24" s="36" t="s">
         <v>33</v>
       </c>
-      <c r="G24" s="95" t="s">
+      <c r="G24" s="36" t="s">
         <v>38</v>
       </c>
-      <c r="H24" s="95"/>
+      <c r="H24" s="36"/>
     </row>
     <row r="25" spans="1:8" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="12"/>
-      <c r="B25" s="12"/>
-      <c r="C25" s="92">
+      <c r="A25" s="67"/>
+      <c r="B25" s="67"/>
+      <c r="C25" s="33">
         <v>22</v>
       </c>
-      <c r="D25" s="93" t="s">
+      <c r="D25" s="34" t="s">
         <v>111</v>
       </c>
-      <c r="E25" s="93" t="s">
+      <c r="E25" s="34" t="s">
         <v>123</v>
       </c>
-      <c r="F25" s="93" t="s">
+      <c r="F25" s="34" t="s">
         <v>72</v>
       </c>
-      <c r="G25" s="93" t="s">
+      <c r="G25" s="34" t="s">
         <v>71</v>
       </c>
-      <c r="H25" s="93"/>
+      <c r="H25" s="34"/>
     </row>
     <row r="26" spans="1:8" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="74"/>
-      <c r="B26" s="74"/>
-      <c r="C26" s="81">
+      <c r="A26" s="15"/>
+      <c r="B26" s="15"/>
+      <c r="C26" s="22">
         <v>23</v>
       </c>
-      <c r="D26" s="87"/>
-      <c r="E26" s="67" t="s">
+      <c r="D26" s="28"/>
+      <c r="E26" s="57" t="s">
         <v>25</v>
       </c>
-      <c r="F26" s="67"/>
-      <c r="G26" s="67"/>
-      <c r="H26" s="67"/>
+      <c r="F26" s="57"/>
+      <c r="G26" s="57"/>
+      <c r="H26" s="57"/>
     </row>
     <row r="27" spans="1:8" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="74"/>
-      <c r="B27" s="74"/>
-      <c r="C27" s="81">
+      <c r="A27" s="15"/>
+      <c r="B27" s="15"/>
+      <c r="C27" s="22">
         <v>24</v>
       </c>
-      <c r="D27" s="87"/>
-      <c r="E27" s="67" t="s">
+      <c r="D27" s="28"/>
+      <c r="E27" s="57" t="s">
         <v>25</v>
       </c>
-      <c r="F27" s="67"/>
-      <c r="G27" s="67"/>
-      <c r="H27" s="67"/>
+      <c r="F27" s="57"/>
+      <c r="G27" s="57"/>
+      <c r="H27" s="57"/>
     </row>
     <row r="28" spans="1:8" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="74"/>
-      <c r="B28" s="74"/>
-      <c r="C28" s="81">
+      <c r="A28" s="15"/>
+      <c r="B28" s="15"/>
+      <c r="C28" s="22">
         <v>25</v>
       </c>
-      <c r="D28" s="87"/>
-      <c r="E28" s="67" t="s">
+      <c r="D28" s="28"/>
+      <c r="E28" s="57" t="s">
         <v>25</v>
       </c>
-      <c r="F28" s="67"/>
-      <c r="G28" s="67"/>
-      <c r="H28" s="67"/>
+      <c r="F28" s="57"/>
+      <c r="G28" s="57"/>
+      <c r="H28" s="57"/>
     </row>
     <row r="29" spans="1:8" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="15" t="s">
+      <c r="A29" s="47" t="s">
         <v>65</v>
       </c>
-      <c r="B29" s="18" t="s">
+      <c r="B29" s="50" t="s">
         <v>93</v>
       </c>
-      <c r="C29" s="96">
+      <c r="C29" s="37">
         <v>26</v>
       </c>
-      <c r="D29" s="97" t="s">
+      <c r="D29" s="38" t="s">
         <v>112</v>
       </c>
-      <c r="E29" s="97" t="s">
+      <c r="E29" s="38" t="s">
         <v>35</v>
       </c>
-      <c r="F29" s="97" t="s">
+      <c r="F29" s="38" t="s">
         <v>54</v>
       </c>
-      <c r="G29" s="97" t="s">
+      <c r="G29" s="38" t="s">
         <v>71</v>
       </c>
-      <c r="H29" s="97"/>
+      <c r="H29" s="38"/>
     </row>
     <row r="30" spans="1:8" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="16"/>
-      <c r="B30" s="19"/>
-      <c r="C30" s="98">
+      <c r="A30" s="48"/>
+      <c r="B30" s="51"/>
+      <c r="C30" s="39">
         <v>27</v>
       </c>
-      <c r="D30" s="99" t="s">
+      <c r="D30" s="40" t="s">
         <v>89</v>
       </c>
-      <c r="E30" s="99" t="s">
+      <c r="E30" s="40" t="s">
         <v>36</v>
       </c>
-      <c r="F30" s="99" t="s">
+      <c r="F30" s="40" t="s">
         <v>72</v>
       </c>
-      <c r="G30" s="99" t="s">
+      <c r="G30" s="40" t="s">
         <v>71</v>
       </c>
-      <c r="H30" s="99"/>
+      <c r="H30" s="40"/>
     </row>
     <row r="31" spans="1:8" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="16"/>
-      <c r="B31" s="19"/>
-      <c r="C31" s="96">
+      <c r="A31" s="48"/>
+      <c r="B31" s="51"/>
+      <c r="C31" s="37">
         <v>28</v>
       </c>
-      <c r="D31" s="97" t="s">
+      <c r="D31" s="38" t="s">
         <v>86</v>
       </c>
-      <c r="E31" s="97" t="s">
+      <c r="E31" s="38" t="s">
         <v>3</v>
       </c>
-      <c r="F31" s="97" t="s">
+      <c r="F31" s="38" t="s">
         <v>30</v>
       </c>
-      <c r="G31" s="97" t="s">
+      <c r="G31" s="38" t="s">
         <v>69</v>
       </c>
-      <c r="H31" s="97" t="s">
+      <c r="H31" s="38" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="32" spans="1:8" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="16"/>
-      <c r="B32" s="19"/>
-      <c r="C32" s="98">
+      <c r="A32" s="48"/>
+      <c r="B32" s="51"/>
+      <c r="C32" s="39">
         <v>29</v>
       </c>
-      <c r="D32" s="99" t="s">
+      <c r="D32" s="40" t="s">
         <v>87</v>
       </c>
-      <c r="E32" s="99" t="s">
+      <c r="E32" s="40" t="s">
         <v>4</v>
       </c>
-      <c r="F32" s="99" t="s">
+      <c r="F32" s="40" t="s">
         <v>72</v>
       </c>
-      <c r="G32" s="99" t="s">
+      <c r="G32" s="40" t="s">
         <v>37</v>
       </c>
-      <c r="H32" s="99"/>
+      <c r="H32" s="40"/>
     </row>
     <row r="33" spans="1:8" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="17"/>
-      <c r="B33" s="20"/>
-      <c r="C33" s="96">
+      <c r="A33" s="49"/>
+      <c r="B33" s="52"/>
+      <c r="C33" s="37">
         <v>30</v>
       </c>
-      <c r="D33" s="97" t="s">
+      <c r="D33" s="38" t="s">
         <v>88</v>
       </c>
-      <c r="E33" s="97" t="s">
+      <c r="E33" s="38" t="s">
         <v>34</v>
       </c>
-      <c r="F33" s="97" t="s">
+      <c r="F33" s="38" t="s">
         <v>72</v>
       </c>
-      <c r="G33" s="97" t="s">
+      <c r="G33" s="38" t="s">
         <v>37</v>
       </c>
-      <c r="H33" s="97"/>
+      <c r="H33" s="38"/>
     </row>
     <row r="34" spans="1:8" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="23" t="s">
+      <c r="A34" s="64" t="s">
         <v>145</v>
       </c>
-      <c r="B34" s="23" t="s">
+      <c r="B34" s="64" t="s">
         <v>146</v>
       </c>
-      <c r="C34" s="88">
+      <c r="C34" s="29">
         <v>31</v>
       </c>
-      <c r="D34" s="89"/>
-      <c r="E34" s="89" t="s">
+      <c r="D34" s="30"/>
+      <c r="E34" s="30" t="s">
         <v>124</v>
       </c>
-      <c r="F34" s="89" t="s">
+      <c r="F34" s="30" t="s">
         <v>54</v>
       </c>
-      <c r="G34" s="89" t="s">
+      <c r="G34" s="30" t="s">
         <v>70</v>
       </c>
-      <c r="H34" s="89" t="s">
+      <c r="H34" s="30" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="35" spans="1:8" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="23"/>
-      <c r="B35" s="23"/>
-      <c r="C35" s="90">
+      <c r="A35" s="64"/>
+      <c r="B35" s="64"/>
+      <c r="C35" s="31">
         <v>32</v>
       </c>
-      <c r="D35" s="91"/>
-      <c r="E35" s="91" t="s">
+      <c r="D35" s="32"/>
+      <c r="E35" s="32" t="s">
         <v>125</v>
       </c>
-      <c r="F35" s="91" t="s">
+      <c r="F35" s="32" t="s">
         <v>54</v>
       </c>
-      <c r="G35" s="91" t="s">
+      <c r="G35" s="32" t="s">
         <v>70</v>
       </c>
-      <c r="H35" s="91" t="s">
+      <c r="H35" s="32" t="s">
         <v>57</v>
       </c>
     </row>
     <row r="36" spans="1:8" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="63" t="s">
+      <c r="A36" s="68" t="s">
         <v>52</v>
       </c>
-      <c r="B36" s="65" t="s">
+      <c r="B36" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="C36" s="100">
+      <c r="C36" s="41">
         <v>33</v>
       </c>
-      <c r="D36" s="101" t="s">
+      <c r="D36" s="42" t="s">
         <v>29</v>
       </c>
-      <c r="E36" s="101" t="s">
+      <c r="E36" s="42" t="s">
         <v>59</v>
       </c>
-      <c r="F36" s="101" t="s">
+      <c r="F36" s="42" t="s">
         <v>60</v>
       </c>
-      <c r="G36" s="101" t="s">
+      <c r="G36" s="42" t="s">
         <v>60</v>
       </c>
-      <c r="H36" s="101" t="s">
+      <c r="H36" s="42" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="37" spans="1:8" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="64"/>
-      <c r="B37" s="74"/>
-      <c r="C37" s="81">
+      <c r="A37" s="69"/>
+      <c r="B37" s="15"/>
+      <c r="C37" s="22">
         <v>34</v>
       </c>
-      <c r="D37" s="87"/>
-      <c r="E37" s="68" t="s">
+      <c r="D37" s="28"/>
+      <c r="E37" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="F37" s="68"/>
-      <c r="G37" s="68"/>
-      <c r="H37" s="68"/>
+      <c r="F37" s="14"/>
+      <c r="G37" s="14"/>
+      <c r="H37" s="14"/>
     </row>
     <row r="38" spans="1:8" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="64"/>
-      <c r="B38" s="74"/>
-      <c r="C38" s="81">
+      <c r="A38" s="69"/>
+      <c r="B38" s="15"/>
+      <c r="C38" s="22">
         <v>35</v>
       </c>
-      <c r="D38" s="87"/>
-      <c r="E38" s="68" t="s">
+      <c r="D38" s="28"/>
+      <c r="E38" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="F38" s="68"/>
-      <c r="G38" s="68"/>
-      <c r="H38" s="68"/>
+      <c r="F38" s="14"/>
+      <c r="G38" s="14"/>
+      <c r="H38" s="14"/>
     </row>
     <row r="39" spans="1:8" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="64"/>
-      <c r="B39" s="74"/>
-      <c r="C39" s="81">
+      <c r="A39" s="69"/>
+      <c r="B39" s="15"/>
+      <c r="C39" s="22">
         <v>36</v>
       </c>
-      <c r="D39" s="87"/>
-      <c r="E39" s="68" t="s">
+      <c r="D39" s="28"/>
+      <c r="E39" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="F39" s="68"/>
-      <c r="G39" s="68"/>
-      <c r="H39" s="68"/>
+      <c r="F39" s="14"/>
+      <c r="G39" s="14"/>
+      <c r="H39" s="14"/>
     </row>
     <row r="40" spans="1:8" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="64"/>
-      <c r="B40" s="74"/>
-      <c r="C40" s="81">
+      <c r="A40" s="69"/>
+      <c r="B40" s="15"/>
+      <c r="C40" s="22">
         <v>37</v>
       </c>
-      <c r="D40" s="87"/>
-      <c r="E40" s="67" t="s">
+      <c r="D40" s="28"/>
+      <c r="E40" s="57" t="s">
         <v>25</v>
       </c>
-      <c r="F40" s="67"/>
-      <c r="G40" s="67"/>
-      <c r="H40" s="67"/>
+      <c r="F40" s="57"/>
+      <c r="G40" s="57"/>
+      <c r="H40" s="57"/>
     </row>
     <row r="41" spans="1:8" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="64"/>
-      <c r="B41" s="65" t="s">
+      <c r="A41" s="69"/>
+      <c r="B41" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="C41" s="100">
+      <c r="C41" s="41">
         <v>38</v>
       </c>
-      <c r="D41" s="101" t="s">
+      <c r="D41" s="42" t="s">
         <v>29</v>
       </c>
-      <c r="E41" s="101" t="s">
+      <c r="E41" s="42" t="s">
         <v>50</v>
       </c>
-      <c r="F41" s="101" t="s">
+      <c r="F41" s="42" t="s">
         <v>29</v>
       </c>
-      <c r="G41" s="101" t="s">
+      <c r="G41" s="42" t="s">
         <v>27</v>
       </c>
-      <c r="H41" s="101"/>
+      <c r="H41" s="42"/>
     </row>
     <row r="42" spans="1:8" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="64"/>
-      <c r="B42" s="74"/>
-      <c r="C42" s="81">
+      <c r="A42" s="69"/>
+      <c r="B42" s="15"/>
+      <c r="C42" s="22">
         <v>39</v>
       </c>
-      <c r="D42" s="87"/>
-      <c r="E42" s="67" t="s">
+      <c r="D42" s="28"/>
+      <c r="E42" s="57" t="s">
         <v>25</v>
       </c>
-      <c r="F42" s="67"/>
-      <c r="G42" s="67"/>
-      <c r="H42" s="67"/>
+      <c r="F42" s="57"/>
+      <c r="G42" s="57"/>
+      <c r="H42" s="57"/>
     </row>
     <row r="43" spans="1:8" ht="11.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="64"/>
-      <c r="B43" s="65" t="s">
+      <c r="A43" s="70"/>
+      <c r="B43" s="12" t="s">
         <v>120</v>
       </c>
-      <c r="C43" s="100">
+      <c r="C43" s="41">
         <v>40</v>
       </c>
-      <c r="D43" s="101" t="s">
+      <c r="D43" s="42" t="s">
         <v>29</v>
       </c>
-      <c r="E43" s="101" t="s">
+      <c r="E43" s="42" t="s">
         <v>50</v>
       </c>
-      <c r="F43" s="101" t="s">
+      <c r="F43" s="42" t="s">
         <v>29</v>
       </c>
-      <c r="G43" s="101" t="s">
+      <c r="G43" s="42" t="s">
         <v>27</v>
       </c>
-      <c r="H43" s="101"/>
+      <c r="H43" s="42"/>
     </row>
   </sheetData>
-  <mergeCells count="25">
+  <mergeCells count="26">
+    <mergeCell ref="E19:H19"/>
+    <mergeCell ref="E22:H22"/>
     <mergeCell ref="E40:H40"/>
     <mergeCell ref="A36:A43"/>
     <mergeCell ref="E42:H42"/>
@@ -2536,23 +2551,22 @@
     <mergeCell ref="E28:H28"/>
     <mergeCell ref="A34:A35"/>
     <mergeCell ref="B34:B35"/>
-    <mergeCell ref="A20:A21"/>
-    <mergeCell ref="B20:B21"/>
-    <mergeCell ref="A23:A25"/>
-    <mergeCell ref="B23:B25"/>
-    <mergeCell ref="E19:H19"/>
-    <mergeCell ref="E22:H22"/>
-    <mergeCell ref="A1:B2"/>
-    <mergeCell ref="C1:G2"/>
     <mergeCell ref="E15:H15"/>
     <mergeCell ref="E14:H14"/>
     <mergeCell ref="E16:H16"/>
     <mergeCell ref="A4:A13"/>
     <mergeCell ref="B4:B13"/>
+    <mergeCell ref="C1:E2"/>
+    <mergeCell ref="F1:G2"/>
     <mergeCell ref="A17:A18"/>
     <mergeCell ref="B17:B18"/>
     <mergeCell ref="A29:A33"/>
     <mergeCell ref="B29:B33"/>
+    <mergeCell ref="A1:B2"/>
+    <mergeCell ref="A20:A21"/>
+    <mergeCell ref="B20:B21"/>
+    <mergeCell ref="A23:A25"/>
+    <mergeCell ref="B23:B25"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2574,86 +2588,89 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="24" t="e" vm="1">
+      <c r="A1" s="53" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="26" t="str">
+      <c r="B1" s="53"/>
+      <c r="C1" s="104" t="str">
         <f>Channels!C1</f>
         <v>Full Band Setup</v>
       </c>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-      <c r="F1" s="26"/>
-      <c r="G1" s="26"/>
-      <c r="H1" s="26"/>
-      <c r="I1" s="26"/>
-      <c r="J1" s="26"/>
-      <c r="K1" s="21" t="str">
+      <c r="D1" s="104"/>
+      <c r="E1" s="104"/>
+      <c r="F1" s="104"/>
+      <c r="G1" s="55" t="str" cm="1">
+        <f t="array" aca="1" ref="G1" ca="1">" (" &amp; _xlfn.TEXTAFTER(CELL("filename", A1), "]") &amp; ")"</f>
+        <v xml:space="preserve"> (Inputs)</v>
+      </c>
+      <c r="H1" s="55"/>
+      <c r="I1" s="103"/>
+      <c r="J1" s="103"/>
+      <c r="K1" s="83" t="str">
         <f>Channels!H1</f>
         <v>🌐 theperfectstrangers.band</v>
       </c>
-      <c r="L1" s="21"/>
-      <c r="M1" s="21"/>
+      <c r="L1" s="83"/>
+      <c r="M1" s="83"/>
       <c r="N1" s="7"/>
       <c r="O1" s="7"/>
       <c r="P1" s="7"/>
     </row>
     <row r="2" spans="1:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="25"/>
-      <c r="B2" s="25"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="26"/>
-      <c r="E2" s="26"/>
-      <c r="F2" s="26"/>
-      <c r="G2" s="26"/>
-      <c r="H2" s="26"/>
-      <c r="I2" s="26"/>
-      <c r="J2" s="26"/>
-      <c r="K2" s="22" t="str">
+      <c r="A2" s="54"/>
+      <c r="B2" s="54"/>
+      <c r="C2" s="105"/>
+      <c r="D2" s="105"/>
+      <c r="E2" s="105"/>
+      <c r="F2" s="105"/>
+      <c r="G2" s="56"/>
+      <c r="H2" s="56"/>
+      <c r="I2" s="103"/>
+      <c r="J2" s="103"/>
+      <c r="K2" s="85" t="str">
         <f ca="1">Channels!H2</f>
-        <v>Date Updated: 2026.01.02</v>
-      </c>
-      <c r="L2" s="22"/>
-      <c r="M2" s="22"/>
+        <v>Date Updated: 2026.01.03</v>
+      </c>
+      <c r="L2" s="85"/>
+      <c r="M2" s="85"/>
     </row>
     <row r="3" spans="1:16" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="31" t="s">
+      <c r="A3" s="74" t="s">
         <v>121</v>
       </c>
-      <c r="B3" s="31"/>
-      <c r="C3" s="31"/>
-      <c r="D3" s="31"/>
-      <c r="E3" s="31"/>
-      <c r="F3" s="31"/>
-      <c r="G3" s="31"/>
-      <c r="H3" s="31"/>
+      <c r="B3" s="74"/>
+      <c r="C3" s="74"/>
+      <c r="D3" s="74"/>
+      <c r="E3" s="74"/>
+      <c r="F3" s="74"/>
+      <c r="G3" s="74"/>
+      <c r="H3" s="74"/>
       <c r="I3" s="2"/>
-      <c r="K3" s="33" t="s">
+      <c r="K3" s="88" t="s">
         <v>16</v>
       </c>
-      <c r="L3" s="33"/>
-      <c r="M3" s="33"/>
+      <c r="L3" s="88"/>
+      <c r="M3" s="88"/>
     </row>
     <row r="4" spans="1:16" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="31" t="s">
+      <c r="A4" s="74" t="s">
         <v>0</v>
       </c>
-      <c r="B4" s="31"/>
-      <c r="C4" s="31"/>
-      <c r="D4" s="31"/>
-      <c r="E4" s="31"/>
-      <c r="F4" s="31"/>
-      <c r="G4" s="31"/>
-      <c r="H4" s="31"/>
+      <c r="B4" s="74"/>
+      <c r="C4" s="74"/>
+      <c r="D4" s="74"/>
+      <c r="E4" s="74"/>
+      <c r="F4" s="74"/>
+      <c r="G4" s="74"/>
+      <c r="H4" s="74"/>
       <c r="I4" s="2"/>
-      <c r="K4" s="44">
+      <c r="K4" s="99">
         <v>1</v>
       </c>
-      <c r="L4" s="34" t="s">
+      <c r="L4" s="89" t="s">
         <v>55</v>
       </c>
-      <c r="M4" s="35"/>
+      <c r="M4" s="90"/>
     </row>
     <row r="5" spans="1:16" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
@@ -2681,57 +2698,57 @@
         <v>8</v>
       </c>
       <c r="I5" s="2"/>
-      <c r="K5" s="45"/>
-      <c r="L5" s="36"/>
-      <c r="M5" s="37"/>
+      <c r="K5" s="100"/>
+      <c r="L5" s="91"/>
+      <c r="M5" s="92"/>
     </row>
     <row r="6" spans="1:16" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="50" t="s">
+      <c r="A6" s="76" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="50" t="s">
+      <c r="B6" s="76" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="50" t="s">
+      <c r="C6" s="76" t="s">
         <v>9</v>
       </c>
-      <c r="D6" s="50" t="s">
+      <c r="D6" s="76" t="s">
         <v>14</v>
       </c>
-      <c r="E6" s="50" t="s">
+      <c r="E6" s="76" t="s">
         <v>10</v>
       </c>
-      <c r="F6" s="50" t="s">
+      <c r="F6" s="76" t="s">
         <v>11</v>
       </c>
-      <c r="G6" s="50" t="s">
+      <c r="G6" s="76" t="s">
         <v>12</v>
       </c>
-      <c r="H6" s="51" t="s">
+      <c r="H6" s="81" t="s">
         <v>13</v>
       </c>
       <c r="I6" s="2"/>
-      <c r="K6" s="42">
+      <c r="K6" s="97">
         <v>2</v>
       </c>
-      <c r="L6" s="38" t="s">
+      <c r="L6" s="93" t="s">
         <v>141</v>
       </c>
-      <c r="M6" s="39"/>
+      <c r="M6" s="94"/>
     </row>
     <row r="7" spans="1:16" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="50"/>
-      <c r="B7" s="50"/>
-      <c r="C7" s="50"/>
-      <c r="D7" s="50"/>
-      <c r="E7" s="50"/>
-      <c r="F7" s="50"/>
-      <c r="G7" s="50"/>
-      <c r="H7" s="52"/>
+      <c r="A7" s="76"/>
+      <c r="B7" s="76"/>
+      <c r="C7" s="76"/>
+      <c r="D7" s="76"/>
+      <c r="E7" s="76"/>
+      <c r="F7" s="76"/>
+      <c r="G7" s="76"/>
+      <c r="H7" s="82"/>
       <c r="I7" s="2"/>
-      <c r="K7" s="43"/>
-      <c r="L7" s="40"/>
-      <c r="M7" s="41"/>
+      <c r="K7" s="98"/>
+      <c r="L7" s="95"/>
+      <c r="M7" s="96"/>
     </row>
     <row r="8" spans="1:16" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="4"/>
@@ -2743,13 +2760,13 @@
       <c r="G8" s="4"/>
       <c r="H8" s="4"/>
       <c r="I8" s="2"/>
-      <c r="K8" s="44">
+      <c r="K8" s="99">
         <v>3</v>
       </c>
-      <c r="L8" s="34" t="s">
+      <c r="L8" s="89" t="s">
         <v>51</v>
       </c>
-      <c r="M8" s="35"/>
+      <c r="M8" s="90"/>
     </row>
     <row r="9" spans="1:16" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
@@ -2777,55 +2794,55 @@
         <v>16</v>
       </c>
       <c r="I9" s="2"/>
-      <c r="K9" s="45"/>
-      <c r="L9" s="36"/>
-      <c r="M9" s="37"/>
+      <c r="K9" s="100"/>
+      <c r="L9" s="91"/>
+      <c r="M9" s="92"/>
     </row>
     <row r="10" spans="1:16" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="51" t="s">
+      <c r="A10" s="81" t="s">
         <v>46</v>
       </c>
-      <c r="B10" s="50" t="s">
+      <c r="B10" s="76" t="s">
         <v>45</v>
       </c>
-      <c r="C10" s="53"/>
-      <c r="D10" s="53"/>
-      <c r="E10" s="53"/>
-      <c r="F10" s="53"/>
-      <c r="G10" s="53"/>
-      <c r="H10" s="53"/>
+      <c r="C10" s="77"/>
+      <c r="D10" s="77"/>
+      <c r="E10" s="77"/>
+      <c r="F10" s="77"/>
+      <c r="G10" s="77"/>
+      <c r="H10" s="77"/>
       <c r="I10" s="2"/>
-      <c r="K10" s="42">
+      <c r="K10" s="97">
         <v>4</v>
       </c>
-      <c r="L10" s="38" t="s">
+      <c r="L10" s="93" t="s">
         <v>142</v>
       </c>
-      <c r="M10" s="39"/>
+      <c r="M10" s="94"/>
     </row>
     <row r="11" spans="1:16" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="52"/>
-      <c r="B11" s="50"/>
-      <c r="C11" s="53"/>
-      <c r="D11" s="53"/>
-      <c r="E11" s="53"/>
-      <c r="F11" s="53"/>
-      <c r="G11" s="53"/>
-      <c r="H11" s="53"/>
+      <c r="A11" s="82"/>
+      <c r="B11" s="76"/>
+      <c r="C11" s="77"/>
+      <c r="D11" s="77"/>
+      <c r="E11" s="77"/>
+      <c r="F11" s="77"/>
+      <c r="G11" s="77"/>
+      <c r="H11" s="77"/>
       <c r="I11" s="2"/>
-      <c r="K11" s="43"/>
-      <c r="L11" s="40"/>
-      <c r="M11" s="41"/>
+      <c r="K11" s="98"/>
+      <c r="L11" s="95"/>
+      <c r="M11" s="96"/>
     </row>
     <row r="12" spans="1:16" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I12" s="2"/>
-      <c r="K12" s="44">
+      <c r="K12" s="99">
         <v>5</v>
       </c>
-      <c r="L12" s="34" t="s">
+      <c r="L12" s="89" t="s">
         <v>143</v>
       </c>
-      <c r="M12" s="35"/>
+      <c r="M12" s="90"/>
     </row>
     <row r="13" spans="1:16" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
@@ -2853,65 +2870,73 @@
         <v>24</v>
       </c>
       <c r="I13" s="2"/>
-      <c r="K13" s="45"/>
-      <c r="L13" s="36"/>
-      <c r="M13" s="37"/>
+      <c r="K13" s="100"/>
+      <c r="L13" s="91"/>
+      <c r="M13" s="92"/>
     </row>
     <row r="14" spans="1:16" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="54" t="s">
+      <c r="A14" s="86" t="s">
         <v>133</v>
       </c>
-      <c r="B14" s="54" t="s">
+      <c r="B14" s="86" t="s">
         <v>134</v>
       </c>
-      <c r="C14" s="53"/>
-      <c r="D14" s="53"/>
-      <c r="E14" s="54" t="s">
+      <c r="C14" s="77"/>
+      <c r="D14" s="77"/>
+      <c r="E14" s="86" t="s">
         <v>49</v>
       </c>
-      <c r="F14" s="54" t="s">
+      <c r="F14" s="86" t="s">
         <v>61</v>
       </c>
-      <c r="G14" s="53"/>
-      <c r="H14" s="54" t="s">
+      <c r="G14" s="77"/>
+      <c r="H14" s="86" t="s">
         <v>120</v>
       </c>
       <c r="I14" s="2"/>
-      <c r="K14" s="42">
+      <c r="K14" s="97">
         <v>6</v>
       </c>
-      <c r="L14" s="38"/>
-      <c r="M14" s="39"/>
+      <c r="L14" s="93"/>
+      <c r="M14" s="94"/>
     </row>
     <row r="15" spans="1:16" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="54"/>
-      <c r="B15" s="54"/>
-      <c r="C15" s="53"/>
-      <c r="D15" s="53"/>
-      <c r="E15" s="54"/>
-      <c r="F15" s="54"/>
-      <c r="G15" s="53"/>
-      <c r="H15" s="54"/>
+      <c r="A15" s="86"/>
+      <c r="B15" s="86"/>
+      <c r="C15" s="77"/>
+      <c r="D15" s="77"/>
+      <c r="E15" s="86"/>
+      <c r="F15" s="86"/>
+      <c r="G15" s="77"/>
+      <c r="H15" s="86"/>
       <c r="I15" s="2"/>
-      <c r="K15" s="43"/>
-      <c r="L15" s="40"/>
-      <c r="M15" s="41"/>
+      <c r="K15" s="98"/>
+      <c r="L15" s="95"/>
+      <c r="M15" s="96"/>
     </row>
     <row r="16" spans="1:16" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I16" s="2"/>
+      <c r="K16" s="99">
+        <v>7</v>
+      </c>
+      <c r="L16" s="89"/>
+      <c r="M16" s="90"/>
     </row>
     <row r="17" spans="1:13" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="31" t="s">
+      <c r="A17" s="74" t="s">
         <v>7</v>
       </c>
-      <c r="B17" s="31"/>
-      <c r="C17" s="31"/>
-      <c r="D17" s="31"/>
-      <c r="E17" s="31"/>
-      <c r="F17" s="31"/>
-      <c r="G17" s="31"/>
-      <c r="H17" s="31"/>
+      <c r="B17" s="74"/>
+      <c r="C17" s="74"/>
+      <c r="D17" s="74"/>
+      <c r="E17" s="74"/>
+      <c r="F17" s="74"/>
+      <c r="G17" s="74"/>
+      <c r="H17" s="74"/>
       <c r="I17" s="6"/>
+      <c r="K17" s="100"/>
+      <c r="L17" s="91"/>
+      <c r="M17" s="92"/>
     </row>
     <row r="18" spans="1:13" ht="14.1" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
@@ -2939,67 +2964,57 @@
         <v>8</v>
       </c>
       <c r="I18" s="2"/>
-      <c r="K18" s="32" t="s">
-        <v>108</v>
-      </c>
-      <c r="L18" s="32"/>
-      <c r="M18" s="32"/>
+      <c r="K18" s="97">
+        <v>8</v>
+      </c>
+      <c r="L18" s="93"/>
+      <c r="M18" s="94"/>
     </row>
     <row r="19" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="49" t="s">
+      <c r="A19" s="71" t="s">
         <v>126</v>
       </c>
-      <c r="B19" s="49" t="s">
+      <c r="B19" s="71" t="s">
         <v>127</v>
       </c>
-      <c r="C19" s="56" t="s">
+      <c r="C19" s="72" t="s">
         <v>138</v>
       </c>
-      <c r="D19" s="56" t="s">
+      <c r="D19" s="72" t="s">
         <v>137</v>
       </c>
-      <c r="E19" s="47" t="s">
+      <c r="E19" s="73" t="s">
         <v>128</v>
       </c>
-      <c r="F19" s="47" t="s">
+      <c r="F19" s="73" t="s">
         <v>129</v>
       </c>
-      <c r="G19" s="61" t="s">
+      <c r="G19" s="84" t="s">
         <v>135</v>
       </c>
-      <c r="H19" s="61" t="s">
+      <c r="H19" s="84" t="s">
         <v>136</v>
       </c>
       <c r="I19" s="2"/>
-      <c r="K19" t="s">
-        <v>97</v>
-      </c>
-      <c r="L19" t="s">
-        <v>98</v>
-      </c>
-      <c r="M19" t="s">
-        <v>107</v>
-      </c>
+      <c r="K19" s="98"/>
+      <c r="L19" s="95"/>
+      <c r="M19" s="96"/>
     </row>
     <row r="20" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="49"/>
-      <c r="B20" s="49"/>
-      <c r="C20" s="56"/>
-      <c r="D20" s="56"/>
-      <c r="E20" s="47"/>
-      <c r="F20" s="47"/>
-      <c r="G20" s="61"/>
-      <c r="H20" s="61"/>
+      <c r="A20" s="71"/>
+      <c r="B20" s="71"/>
+      <c r="C20" s="72"/>
+      <c r="D20" s="72"/>
+      <c r="E20" s="73"/>
+      <c r="F20" s="73"/>
+      <c r="G20" s="84"/>
+      <c r="H20" s="84"/>
       <c r="I20" s="2"/>
-      <c r="K20" t="s">
-        <v>103</v>
-      </c>
-      <c r="L20" t="s">
-        <v>99</v>
-      </c>
-      <c r="M20" t="s">
-        <v>100</v>
-      </c>
+      <c r="K20" s="99">
+        <v>9</v>
+      </c>
+      <c r="L20" s="89"/>
+      <c r="M20" s="90"/>
     </row>
     <row r="21" spans="1:13" ht="14.1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="5"/>
@@ -3011,71 +3026,51 @@
       <c r="G21" s="5"/>
       <c r="H21" s="5"/>
       <c r="I21" s="2"/>
-      <c r="K21" t="s">
-        <v>104</v>
-      </c>
-      <c r="L21" t="s">
-        <v>99</v>
-      </c>
-      <c r="M21" t="s">
-        <v>100</v>
-      </c>
+      <c r="K21" s="100"/>
+      <c r="L21" s="91"/>
+      <c r="M21" s="92"/>
     </row>
     <row r="22" spans="1:13" ht="14.1" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="I22" s="2"/>
-      <c r="K22" t="s">
-        <v>105</v>
-      </c>
-      <c r="L22" t="s">
-        <v>99</v>
-      </c>
-      <c r="M22" t="s">
-        <v>100</v>
-      </c>
+      <c r="K22" s="97">
+        <v>10</v>
+      </c>
+      <c r="L22" s="93"/>
+      <c r="M22" s="94"/>
     </row>
     <row r="23" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="31" t="s">
+      <c r="A23" s="74" t="s">
         <v>122</v>
       </c>
-      <c r="B23" s="31"/>
-      <c r="C23" s="31"/>
-      <c r="D23" s="31"/>
-      <c r="E23" s="31"/>
-      <c r="F23" s="31"/>
-      <c r="G23" s="31"/>
-      <c r="H23" s="31"/>
+      <c r="B23" s="74"/>
+      <c r="C23" s="74"/>
+      <c r="D23" s="74"/>
+      <c r="E23" s="74"/>
+      <c r="F23" s="74"/>
+      <c r="G23" s="74"/>
+      <c r="H23" s="74"/>
       <c r="I23" s="2"/>
-      <c r="K23" t="s">
-        <v>106</v>
-      </c>
-      <c r="L23" t="s">
-        <v>101</v>
-      </c>
-      <c r="M23" t="s">
-        <v>102</v>
-      </c>
+      <c r="K23" s="98"/>
+      <c r="L23" s="95"/>
+      <c r="M23" s="96"/>
     </row>
     <row r="24" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="31" t="s">
+      <c r="A24" s="74" t="s">
         <v>0</v>
       </c>
-      <c r="B24" s="31"/>
-      <c r="C24" s="31"/>
-      <c r="D24" s="31"/>
-      <c r="E24" s="31"/>
-      <c r="F24" s="31"/>
-      <c r="G24" s="31"/>
-      <c r="H24" s="31"/>
+      <c r="B24" s="74"/>
+      <c r="C24" s="74"/>
+      <c r="D24" s="74"/>
+      <c r="E24" s="74"/>
+      <c r="F24" s="74"/>
+      <c r="G24" s="74"/>
+      <c r="H24" s="74"/>
       <c r="I24" s="2"/>
-      <c r="K24" t="s">
-        <v>119</v>
-      </c>
-      <c r="L24" t="s">
-        <v>99</v>
-      </c>
-      <c r="M24" t="s">
-        <v>100</v>
-      </c>
+      <c r="K24" s="99">
+        <v>11</v>
+      </c>
+      <c r="L24" s="89"/>
+      <c r="M24" s="90"/>
     </row>
     <row r="25" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
@@ -3103,52 +3098,63 @@
         <v>8</v>
       </c>
       <c r="I25" s="2"/>
+      <c r="K25" s="100"/>
+      <c r="L25" s="91"/>
+      <c r="M25" s="92"/>
     </row>
     <row r="26" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="55" t="s">
+      <c r="A26" s="101" t="s">
         <v>114</v>
       </c>
-      <c r="B26" s="49" t="s">
+      <c r="B26" s="71" t="s">
         <v>115</v>
       </c>
-      <c r="C26" s="56" t="s">
+      <c r="C26" s="72" t="s">
         <v>39</v>
       </c>
-      <c r="D26" s="56" t="s">
+      <c r="D26" s="72" t="s">
         <v>53</v>
       </c>
-      <c r="E26" s="47" t="s">
+      <c r="E26" s="73" t="s">
         <v>1</v>
       </c>
-      <c r="F26" s="47" t="s">
+      <c r="F26" s="73" t="s">
         <v>2</v>
       </c>
-      <c r="G26" s="47" t="s">
+      <c r="G26" s="73" t="s">
         <v>123</v>
       </c>
-      <c r="H26" s="53"/>
+      <c r="H26" s="77"/>
       <c r="I26" s="2"/>
+      <c r="K26" s="97">
+        <v>12</v>
+      </c>
+      <c r="L26" s="93"/>
+      <c r="M26" s="94"/>
     </row>
     <row r="27" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="57"/>
-      <c r="B27" s="49"/>
-      <c r="C27" s="56"/>
-      <c r="D27" s="56"/>
-      <c r="E27" s="47"/>
-      <c r="F27" s="47"/>
-      <c r="G27" s="47"/>
-      <c r="H27" s="53"/>
+      <c r="A27" s="102"/>
+      <c r="B27" s="71"/>
+      <c r="C27" s="72"/>
+      <c r="D27" s="72"/>
+      <c r="E27" s="73"/>
+      <c r="F27" s="73"/>
+      <c r="G27" s="73"/>
+      <c r="H27" s="77"/>
       <c r="I27" s="2"/>
+      <c r="K27" s="98"/>
+      <c r="L27" s="95"/>
+      <c r="M27" s="96"/>
     </row>
     <row r="28" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="48"/>
-      <c r="B28" s="48"/>
-      <c r="C28" s="48"/>
-      <c r="D28" s="48"/>
-      <c r="E28" s="48"/>
-      <c r="F28" s="48"/>
-      <c r="G28" s="48"/>
-      <c r="H28" s="48"/>
+      <c r="A28" s="11"/>
+      <c r="B28" s="11"/>
+      <c r="C28" s="11"/>
+      <c r="D28" s="11"/>
+      <c r="E28" s="11"/>
+      <c r="F28" s="11"/>
+      <c r="G28" s="11"/>
+      <c r="H28" s="11"/>
       <c r="I28" s="2"/>
     </row>
     <row r="29" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
@@ -3177,60 +3183,101 @@
         <v>16</v>
       </c>
       <c r="I29" s="2"/>
+      <c r="K29" s="87" t="s">
+        <v>108</v>
+      </c>
+      <c r="L29" s="87"/>
+      <c r="M29" s="87"/>
     </row>
     <row r="30" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="53"/>
-      <c r="B30" s="58" t="s">
+      <c r="A30" s="77"/>
+      <c r="B30" s="78" t="s">
         <v>5</v>
       </c>
-      <c r="C30" s="58" t="s">
+      <c r="C30" s="78" t="s">
         <v>6</v>
       </c>
-      <c r="D30" s="58" t="s">
+      <c r="D30" s="78" t="s">
         <v>3</v>
       </c>
-      <c r="E30" s="58" t="s">
+      <c r="E30" s="78" t="s">
         <v>4</v>
       </c>
-      <c r="F30" s="58" t="s">
+      <c r="F30" s="78" t="s">
         <v>65</v>
       </c>
-      <c r="G30" s="59" t="s">
+      <c r="G30" s="80" t="s">
         <v>124</v>
       </c>
-      <c r="H30" s="59" t="s">
+      <c r="H30" s="80" t="s">
         <v>125</v>
       </c>
       <c r="I30" s="2"/>
+      <c r="K30" t="s">
+        <v>97</v>
+      </c>
+      <c r="L30" t="s">
+        <v>98</v>
+      </c>
+      <c r="M30" t="s">
+        <v>107</v>
+      </c>
     </row>
     <row r="31" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="53"/>
-      <c r="B31" s="60"/>
-      <c r="C31" s="60"/>
-      <c r="D31" s="60"/>
-      <c r="E31" s="60"/>
-      <c r="F31" s="60"/>
-      <c r="G31" s="59"/>
-      <c r="H31" s="59"/>
+      <c r="A31" s="77"/>
+      <c r="B31" s="79"/>
+      <c r="C31" s="79"/>
+      <c r="D31" s="79"/>
+      <c r="E31" s="79"/>
+      <c r="F31" s="79"/>
+      <c r="G31" s="80"/>
+      <c r="H31" s="80"/>
       <c r="I31" s="2"/>
+      <c r="K31" t="s">
+        <v>103</v>
+      </c>
+      <c r="L31" t="s">
+        <v>99</v>
+      </c>
+      <c r="M31" t="s">
+        <v>100</v>
+      </c>
     </row>
     <row r="32" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="I32" s="2"/>
-    </row>
-    <row r="33" spans="1:9" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="31" t="s">
+      <c r="K32" t="s">
+        <v>104</v>
+      </c>
+      <c r="L32" t="s">
+        <v>99</v>
+      </c>
+      <c r="M32" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="33" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="74" t="s">
         <v>7</v>
       </c>
-      <c r="B33" s="31"/>
-      <c r="C33" s="31"/>
-      <c r="D33" s="31"/>
-      <c r="E33" s="31"/>
-      <c r="F33" s="31"/>
-      <c r="G33" s="31"/>
-      <c r="H33" s="31"/>
+      <c r="B33" s="74"/>
+      <c r="C33" s="74"/>
+      <c r="D33" s="74"/>
+      <c r="E33" s="74"/>
+      <c r="F33" s="74"/>
+      <c r="G33" s="74"/>
+      <c r="H33" s="74"/>
       <c r="I33" s="2"/>
-    </row>
-    <row r="34" spans="1:9" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="K33" t="s">
+        <v>105</v>
+      </c>
+      <c r="L33" t="s">
+        <v>99</v>
+      </c>
+      <c r="M33" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="34" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
         <v>1</v>
       </c>
@@ -3256,43 +3303,71 @@
         <v>8</v>
       </c>
       <c r="I34" s="2"/>
-    </row>
-    <row r="35" spans="1:9" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="50" t="s">
+      <c r="K34" t="s">
+        <v>106</v>
+      </c>
+      <c r="L34" t="s">
+        <v>101</v>
+      </c>
+      <c r="M34" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="35" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="76" t="s">
         <v>130</v>
       </c>
-      <c r="B35" s="50" t="s">
+      <c r="B35" s="76" t="s">
         <v>131</v>
       </c>
-      <c r="C35" s="53"/>
-      <c r="D35" s="53"/>
-      <c r="E35" s="62" t="s">
+      <c r="C35" s="77"/>
+      <c r="D35" s="77"/>
+      <c r="E35" s="75" t="s">
         <v>132</v>
       </c>
-      <c r="F35" s="62" t="s">
+      <c r="F35" s="75" t="s">
         <v>139</v>
       </c>
-      <c r="G35" s="62" t="s">
+      <c r="G35" s="75" t="s">
         <v>116</v>
       </c>
-      <c r="H35" s="62" t="s">
+      <c r="H35" s="75" t="s">
         <v>140</v>
       </c>
       <c r="I35" s="2"/>
-    </row>
-    <row r="36" spans="1:9" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="50"/>
-      <c r="B36" s="50"/>
-      <c r="C36" s="53"/>
-      <c r="D36" s="53"/>
-      <c r="E36" s="62"/>
-      <c r="F36" s="62"/>
-      <c r="G36" s="62"/>
-      <c r="H36" s="62"/>
+      <c r="K35" t="s">
+        <v>119</v>
+      </c>
+      <c r="L35" t="s">
+        <v>99</v>
+      </c>
+      <c r="M35" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="36" spans="1:13" ht="14.1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="76"/>
+      <c r="B36" s="76"/>
+      <c r="C36" s="77"/>
+      <c r="D36" s="77"/>
+      <c r="E36" s="75"/>
+      <c r="F36" s="75"/>
+      <c r="G36" s="75"/>
+      <c r="H36" s="75"/>
       <c r="I36" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="80">
+  <mergeCells count="93">
+    <mergeCell ref="K24:K25"/>
+    <mergeCell ref="L24:M25"/>
+    <mergeCell ref="K26:K27"/>
+    <mergeCell ref="L26:M27"/>
+    <mergeCell ref="K18:K19"/>
+    <mergeCell ref="L18:M19"/>
+    <mergeCell ref="K20:K21"/>
+    <mergeCell ref="L20:M21"/>
+    <mergeCell ref="K22:K23"/>
+    <mergeCell ref="L22:M23"/>
     <mergeCell ref="G14:G15"/>
     <mergeCell ref="H14:H15"/>
     <mergeCell ref="F26:F27"/>
@@ -3301,7 +3376,15 @@
     <mergeCell ref="D14:D15"/>
     <mergeCell ref="E14:E15"/>
     <mergeCell ref="F14:F15"/>
-    <mergeCell ref="K18:M18"/>
+    <mergeCell ref="B26:B27"/>
+    <mergeCell ref="C26:C27"/>
+    <mergeCell ref="D26:D27"/>
+    <mergeCell ref="A17:H17"/>
+    <mergeCell ref="F19:F20"/>
+    <mergeCell ref="A26:A27"/>
+    <mergeCell ref="A23:H23"/>
+    <mergeCell ref="A24:H24"/>
+    <mergeCell ref="K29:M29"/>
     <mergeCell ref="K3:M3"/>
     <mergeCell ref="L4:M5"/>
     <mergeCell ref="L6:M7"/>
@@ -3315,6 +3398,8 @@
     <mergeCell ref="L12:M13"/>
     <mergeCell ref="K14:K15"/>
     <mergeCell ref="L14:M15"/>
+    <mergeCell ref="K16:K17"/>
+    <mergeCell ref="L16:M17"/>
     <mergeCell ref="K1:M1"/>
     <mergeCell ref="C10:C11"/>
     <mergeCell ref="D10:D11"/>
@@ -3331,11 +3416,7 @@
     <mergeCell ref="F6:F7"/>
     <mergeCell ref="K2:M2"/>
     <mergeCell ref="A14:A15"/>
-    <mergeCell ref="B26:B27"/>
-    <mergeCell ref="C26:C27"/>
-    <mergeCell ref="D26:D27"/>
     <mergeCell ref="A1:B2"/>
-    <mergeCell ref="C1:J2"/>
     <mergeCell ref="G6:G7"/>
     <mergeCell ref="H6:H7"/>
     <mergeCell ref="H10:H11"/>
@@ -3343,9 +3424,8 @@
     <mergeCell ref="B10:B11"/>
     <mergeCell ref="G10:G11"/>
     <mergeCell ref="F10:F11"/>
-    <mergeCell ref="A17:H17"/>
-    <mergeCell ref="F19:F20"/>
-    <mergeCell ref="A26:A27"/>
+    <mergeCell ref="C1:F2"/>
+    <mergeCell ref="G1:H2"/>
     <mergeCell ref="A30:A31"/>
     <mergeCell ref="B30:B31"/>
     <mergeCell ref="C30:C31"/>
@@ -3366,8 +3446,6 @@
     <mergeCell ref="D35:D36"/>
     <mergeCell ref="E35:E36"/>
     <mergeCell ref="F35:F36"/>
-    <mergeCell ref="A23:H23"/>
-    <mergeCell ref="A24:H24"/>
     <mergeCell ref="A19:A20"/>
     <mergeCell ref="B19:B20"/>
     <mergeCell ref="C19:C20"/>

</xml_diff>